<commit_message>
feat(map): unify district cluster architecture, standardize Tseung Kwan O, add Chai Wan profile, and update minibus transit notes
</commit_message>
<xml_diff>
--- a/导出方案项目描述库.xlsx
+++ b/导出方案项目描述库.xlsx
@@ -579,7 +579,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>九龙塘低密度豪宅区 / 广播道及毕架山</t>
+          <t>九龙塘及毕架山</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1600米(约19分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁九龍塘站约1600米(约19分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>九龙塘低密度豪宅区 / 广播道及毕架山</t>
+          <t>九龙塘及毕架山</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1446米(约17分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁九龍塘站约1446米(约17分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共14伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -704,7 +704,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>九龙塘低密度豪宅区 / 广播道及毕架山</t>
+          <t>九龙塘及毕架山</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1446米(约17分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁九龍塘站约1446米(约17分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共46伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -767,7 +767,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>九龙塘低密度豪宅区 / 广播道及毕架山</t>
+          <t>九龙塘及毕架山</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1403米(约16分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁九龍塘站约1403米(约16分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>九龙塘低密度豪宅区 / 广播道及毕架山</t>
+          <t>九龙塘及毕架山</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁天后站约2297米(约27分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁天后站约2297米(约27分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共4伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -934,7 +934,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁長沙灣站约2210米(约26分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁長沙灣站约2210米(约26分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约1070米(约12分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁旺角東站约1070米(约12分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共110伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约606米(约7分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁旺角東站约606米(约7分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共165伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约724米(约8分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁旺角東站约724米(约8分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约1165米(约14分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁土瓜灣站约1165米(约14分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1371,7 +1371,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约1030米(约12分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁旺角東站约1030米(约12分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共80伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约740米(约8分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁旺角東站约740米(约8分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共75伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约1090米(约13分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁旺角東站约1090米(约13分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共18伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约1115米(约13分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁土瓜灣站约1115米(约13分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共14伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约554米(约6分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁旺角東站约554米(约6分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共71伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -1996,7 +1996,7 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约971米(约11分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁旺角東站约971米(约11分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共56伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁宋皇臺站约1045米(约12分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁宋皇臺站约1045米(约12分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共45伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -2080,7 +2080,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -2647,7 +2647,7 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -2710,7 +2710,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -2773,7 +2773,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -2962,7 +2962,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -3025,7 +3025,7 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -3151,7 +3151,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -3214,7 +3214,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -3340,7 +3340,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -3403,7 +3403,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -3529,7 +3529,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -3655,7 +3655,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -3781,7 +3781,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -3949,7 +3949,7 @@
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁深水埗站约836米(约10分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁深水埗站约836米(约10分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为32校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁奧運站约909米(约10分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁奧運站约909米(约10分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为32校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4138,7 +4138,7 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁奧運站约909米(约10分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁奧運站约909米(约10分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为32校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角站约819米(约9分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁旺角站约819米(约9分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为32校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4327,7 +4327,7 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁長沙灣站约2071米(约24分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁長沙灣站约2071米(约24分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1019米(约12分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁九龍塘站约1019米(约12分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4453,7 +4453,7 @@
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁何文田站约550米(约6分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁何文田站约550米(约6分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约724米(约8分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁土瓜灣站约724米(约8分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约724米(约8分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁土瓜灣站约724米(约8分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4831,7 +4831,7 @@
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约648米(约7分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁土瓜灣站约648米(约7分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4894,7 +4894,7 @@
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约598米(约7分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁土瓜灣站约598米(约7分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁何文田站约599米(约7分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁何文田站约599米(约7分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -5020,7 +5020,7 @@
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁荔枝角站约874米(约10分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁荔枝角站约874米(约10分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -5083,7 +5083,7 @@
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁南昌站约571米(约6分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁南昌站约571米(约6分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -5146,7 +5146,7 @@
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁南昌站约1374米(约16分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁南昌站约1374米(约16分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为40校网 / 深水埗区校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁宋皇臺站约559米(约6分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁宋皇臺站约559米(约6分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共92伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -5417,7 +5417,7 @@
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>北角核心及炮台山</t>
+          <t>北角及炮台山</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>北角核心及炮台山</t>
+          <t>北角及炮台山</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>北角核心及炮台山</t>
+          <t>北角及炮台山</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
@@ -5605,7 +5605,7 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>北角核心及炮台山</t>
+          <t>北角及炮台山</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁北角站约661米(约7分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁北角站约661米(约7分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为14校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -5668,7 +5668,7 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>北角核心及炮台山</t>
+          <t>北角及炮台山</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
@@ -5730,7 +5730,7 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>北角核心及炮台山</t>
+          <t>北角及炮台山</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>北角核心及炮台山</t>
+          <t>北角及炮台山</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
@@ -5896,7 +5896,7 @@
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁中環站约734米(约8分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁中環站约734米(约8分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共99伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -5959,7 +5959,7 @@
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁灣仔站约1708米(约20分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁灣仔站约1708米(约20分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L87" s="3" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁灣仔站约1708米(约20分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁灣仔站约1708米(约20分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共19伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -6084,7 +6084,7 @@
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁金鐘站约1709米(约20分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁金鐘站约1709米(约20分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L89" s="3" t="inlineStr">
@@ -6146,7 +6146,7 @@
       </c>
       <c r="K90" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁香港大學站约1152米(约13分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁香港大學站约1152米(约13分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共7伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -6209,7 +6209,7 @@
       </c>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约891米(约10分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁上環站约891米(约10分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共85伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -6272,7 +6272,7 @@
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁香港大學站约1021米(约12分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁香港大學站约1021米(约12分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L92" s="3" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约947米(约11分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁上環站约947米(约11分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共106伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -6397,7 +6397,7 @@
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约947米(约11分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁上環站约947米(约11分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共66伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -6460,7 +6460,7 @@
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁香港大學站约1241米(约14分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁香港大學站约1241米(约14分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共16伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -6523,7 +6523,7 @@
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约1146米(约13分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁上環站约1146米(约13分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共90伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -6586,7 +6586,7 @@
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁金鐘站约1764米(约21分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁金鐘站约1764米(约21分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L97" s="3" t="inlineStr">
@@ -6648,7 +6648,7 @@
       </c>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁西營盤站约650米(约7分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁西營盤站约650米(约7分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L98" s="3" t="inlineStr">
@@ -7527,7 +7527,7 @@
       </c>
       <c r="K112" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁柴灣站约945米(约11分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁柴灣站约945米(约11分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为16校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -7590,7 +7590,7 @@
       </c>
       <c r="K113" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁天后站约1809米(约21分钟)，雨季建议接驳小巴</t>
+          <t>【交通】步行至最近港铁天后站约1809米(约21分钟)，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L113" s="3" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="K114" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁灣仔站约715米(约8分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁灣仔站约715米(约8分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共167伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -7673,7 +7673,7 @@
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
-          <t>西湾河 / 筲箕湾及阿公岩</t>
+          <t>西湾河及筲箕湾</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
@@ -7736,7 +7736,7 @@
       </c>
       <c r="C116" s="3" t="inlineStr">
         <is>
-          <t>西湾河 / 筲箕湾及阿公岩</t>
+          <t>西湾河及筲箕湾</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
@@ -7799,7 +7799,7 @@
       </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
-          <t>西湾河 / 筲箕湾及阿公岩</t>
+          <t>西湾河及筲箕湾</t>
         </is>
       </c>
       <c r="D117" s="3" t="inlineStr">
@@ -7841,7 +7841,7 @@
       </c>
       <c r="K117" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁筲箕灣站约1073米(约12分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁筲箕灣站约1073米(约12分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为16校网 / 东区校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -7904,7 +7904,7 @@
       </c>
       <c r="K118" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁堅尼地城站约1541米(约18分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁堅尼地城站约1541米(约18分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -7925,7 +7925,7 @@
       </c>
       <c r="C119" s="3" t="inlineStr">
         <is>
-          <t>西营盘及石塘咀 / 上环</t>
+          <t>上环及西营盘</t>
         </is>
       </c>
       <c r="D119" s="3" t="inlineStr">
@@ -7988,7 +7988,7 @@
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>西营盘及石塘咀 / 上环</t>
+          <t>上环及西营盘</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
@@ -8030,7 +8030,7 @@
       </c>
       <c r="K120" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约555米(约6分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁上環站约555米(约6分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共13伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -8679,7 +8679,7 @@
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>鸭脷洲 (海怡半岛及鸭脷洲大街)</t>
+          <t>鸭脷洲</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
@@ -8742,7 +8742,7 @@
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>鸭脷洲 (海怡半岛及鸭脷洲大街)</t>
+          <t>鸭脷洲</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="K133" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁黃竹坑站约624米(约7分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁黃竹坑站约624米(约7分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -9117,7 +9117,7 @@
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>鸭脷洲 (海怡半岛及鸭脷洲大街)</t>
+          <t>鸭脷洲</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
@@ -9159,7 +9159,7 @@
       </c>
       <c r="K138" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁利東站约892米(约10分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁利東站约892米(约10分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -9180,7 +9180,7 @@
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>鸭脷洲 (海怡半岛及鸭脷洲大街)</t>
+          <t>鸭脷洲</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
@@ -9305,7 +9305,7 @@
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>鸭脷洲 (海怡半岛及鸭脷洲大街)</t>
+          <t>鸭脷洲</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="K141" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁海怡半島站约594米(约7分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁海怡半島站约594米(约7分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -9410,7 +9410,7 @@
       </c>
       <c r="K142" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁銅鑼灣站约1891米(约22分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁銅鑼灣站约1891米(约22分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共156伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -9473,7 +9473,7 @@
       </c>
       <c r="K143" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁銅鑼灣站约1824米(约21分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁銅鑼灣站约1824米(约21分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共18伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -9536,7 +9536,7 @@
       </c>
       <c r="K144" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁黃竹坑站约598米(约7分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁黃竹坑站约598米(约7分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -9557,7 +9557,7 @@
       </c>
       <c r="C145" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D145" s="3" t="inlineStr">
@@ -9620,7 +9620,7 @@
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
@@ -9788,7 +9788,7 @@
       </c>
       <c r="K148" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁南昌站约1247米(约15分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁南昌站约1247米(约15分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为40校网 / 深水埗区校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -10039,7 +10039,7 @@
       </c>
       <c r="K152" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁柴灣站约945米(约11分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁柴灣站约945米(约11分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为16校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -10102,7 +10102,7 @@
       </c>
       <c r="K153" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁長沙灣站约817米(约10分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁長沙灣站约817米(约10分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -10228,7 +10228,7 @@
       </c>
       <c r="K155" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁灣仔站约1065米(约13分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁灣仔站约1065米(约13分钟)，建议接驳小巴至地铁 ；
 【社区】单幢式精致大厦(共24伙)，内部公用绿化及大型会所设施相对小巧</t>
         </is>
       </c>
@@ -10249,7 +10249,7 @@
       </c>
       <c r="C156" s="3" t="inlineStr">
         <is>
-          <t>将军澳南及日出康城</t>
+          <t>将军澳及日出康城</t>
         </is>
       </c>
       <c r="D156" s="3" t="inlineStr">
@@ -10312,7 +10312,7 @@
       </c>
       <c r="C157" s="3" t="inlineStr">
         <is>
-          <t>将军澳南及日出康城</t>
+          <t>将军澳及日出康城</t>
         </is>
       </c>
       <c r="D157" s="3" t="inlineStr">
@@ -10375,7 +10375,7 @@
       </c>
       <c r="C158" s="3" t="inlineStr">
         <is>
-          <t>北角核心及炮台山</t>
+          <t>北角及炮台山</t>
         </is>
       </c>
       <c r="D158" s="3" t="inlineStr">
@@ -10480,7 +10480,7 @@
       </c>
       <c r="K159" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁太子站约1028米(约12分钟)，雨季建议接驳小巴 ；
+          <t>【交通】步行至最近港铁太子站约1028米(约12分钟)，建议接驳小巴至地铁 ；
 【校网】所属公立校网为32校网 / 油尖旺区校网，重视升学建议结合片区优质私立或国际学校</t>
         </is>
       </c>
@@ -10501,7 +10501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10561,7 +10561,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>启德城中心 (AIRSIDE/天玺) / 启德跑道区</t>
+          <t>启德城中心 / 启德跑道区</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -10666,7 +10666,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>九龙塘低密度豪宅区 / 广播道及毕架山</t>
+          <t>九龙塘及毕架山</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -10771,7 +10771,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>鸭脷洲 (海怡半岛及鸭脷洲大街)</t>
+          <t>鸭脷洲</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -11016,7 +11016,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>石澳、大浪湾及鹤咀</t>
+          <t>石澳及鹤咀</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -11051,7 +11051,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>山顶 (The Peak)</t>
+          <t>山顶</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -11086,7 +11086,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>中半山 (Mid-Levels Central)</t>
+          <t>中半山</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>西半山 (Mid-Levels West)</t>
+          <t>西半山</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -11156,7 +11156,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>坚尼地城 (Kennedy Town)</t>
+          <t>坚尼地城</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -11191,7 +11191,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>西营盘及石塘咀 / 上环</t>
+          <t>上环及西营盘</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -11436,7 +11436,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>东半山 (Mid-Levels East)</t>
+          <t>东半山</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -11506,7 +11506,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>湾仔核心区</t>
+          <t>湾仔</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -11541,7 +11541,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>北角核心及炮台山</t>
+          <t>北角及炮台山</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -11611,7 +11611,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>西湾河 / 筲箕湾及阿公岩</t>
+          <t>西湾河及筲箕湾</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -11681,7 +11681,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>将军澳南及日出康城</t>
+          <t>将军澳及日出康城</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -11702,6 +11702,41 @@
       <c r="G34" s="3" t="inlineStr">
         <is>
           <t>未来将军澳第 137 区超大规模综合社区规划与跨湾水上交通网络落地，巩固其作为现代智能化滨海生活典范的活力前景。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>六、港岛东区</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>柴湾及小西湾</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>港岛东沿海成熟居住绿核，港铁港岛线东端始发站与蓝筹临海社区生活圈。</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>柴湾早年因盛产木柴烧炭而得名，曾为客家传统村落；20 世纪下半叶随港铁港岛线通车及填海工程全面蜕变，小西湾自 1990 年代发展为高质素临海中产住宅区，兼具山海生态与现代化配套。</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>港岛东极具自住性价比与高生活便利度的成熟纯住区。既享港岛线始发站直达中环金钟的通勤优势，又拥有小西湾海滨长廊、蓝湾半岛滨水生活圈与大片城市绿荫。</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>柴湾旧工厦与工业用地持续活化升级，全新优质住宅项目（如海德园等）陆续入市推动片区人居面貌与环境品质显著跃升。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(export): deploy 5D value & trade-off system, strict dimension ordering, card-row layout, and MTR on-top corrections
</commit_message>
<xml_diff>
--- a/导出方案项目描述库.xlsx
+++ b/导出方案项目描述库.xlsx
@@ -616,12 +616,16 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖41校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 九龙塘龙庭里8号超级豪宅巅峰之作
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1600米(约19分钟)，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -678,13 +682,16 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖41校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 九龙塘龙庭里8号超级豪宅巅峰之作
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1446米(约17分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共14伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -741,13 +748,16 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖41校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 九龙塘龙庭里8号超级豪宅巅峰之作
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1446米(约17分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共46伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -804,12 +814,16 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖41校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 九龙塘广播道半山珍稀向南大宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1403米(约16分钟)，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
@@ -866,13 +880,16 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖41校网 / 九龙城区校网名校网 ｜ 现楼</t>
+          <t>★ 九龙塘喇沙利道32-38号喇沙小学正对面
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁天后站约2297米(约27分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共4伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -929,13 +946,16 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 嘉里建设精工品质保障</t>
+          <t>★ 九龙笔架山半山龙驹道超级豪宅巅峰
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁長沙灣站约2210米(约26分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🚇【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -992,12 +1012,16 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>港铁九龍站上盖/极速步行直达 ｜ 现楼</t>
+          <t>★ 九龙站上盖香港地标级顶奢天际豪宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁九龙站正上盖 / 直通（直通圆方 ELEMENTS 与九龙站/柯士甸）
+🛍️【商业】基座直通圆方 ELEMENTS 超大型购物中心
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为31校网 / 油尖旺区校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1054,13 +1078,16 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 何文田窝打老道黄金名校地段
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约1070米(约12分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共110伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -1117,12 +1144,16 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 紧邻港铁旺角東站高效通勤</t>
+          <t>★ 太子道西核心地段新鸿基品质力作
+🚇【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>【社区】单幢式精致大厦(共101伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
@@ -1179,13 +1210,16 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 何文田自由道万科品质轻奢地标
+🚇【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约606米(约7分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共165伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -1242,12 +1276,17 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龙城区校网名校网 ｜ 现楼</t>
+          <t>★ 何文田加多利山百年名门显赫地段
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约724米(约8分钟)，建议接驳小巴至地铁</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
@@ -1304,12 +1343,16 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 何文田核心传统豪宅区现楼大宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约1165米(约14分钟)，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1366,13 +1409,16 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 太子道西266号传统豪宅名门腹地
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约1030米(约12分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共80伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -1429,12 +1475,17 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龙城区校网名校网 ｜ 紧邻港铁何文田站高效通勤</t>
+          <t>★ 何文田佛光街23号新鸿基巅峰豪宅标杆
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>【房源】高楼层优质采光单位余货稀缺，推售现场需尽早锁定心仪朝向</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -1491,13 +1542,16 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 九龙顶尖34名校网黄金护城河
+🚇【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约740米(约8分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共75伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
@@ -1554,13 +1608,16 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 太子道西279号极低密名门大宅
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约1090米(约13分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共18伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -1617,12 +1674,16 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龙城区校网名校网 ｜ 紧邻港铁何文田站高效通勤</t>
+          <t>★ 港铁何文田站纯正铁路上盖绝版压轴大盘
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>【交付】属预售楼花阶段(即将发售)，需等待工程竣工后交付</t>
+          <t>⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
@@ -1679,12 +1740,16 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龙城区校网名校网 ｜ 紧邻港铁何文田站高效通勤</t>
+          <t>★ 港铁何文田站纯正铁路上盖绝版压轴大盘
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>【交付】属预售楼花阶段(即将发售)，需等待工程竣工后交付</t>
+          <t>⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
@@ -1741,12 +1806,17 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 紧邻港铁何文田站高效通勤</t>
+          <t>★ 纯正铁路上盖双线枢纽极速通达
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>【交付】属预售楼花阶段(2025年入伙)，需等待工程竣工后交付</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
@@ -1803,12 +1873,17 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 港铁何文田站上盖/极速步行直达</t>
+          <t>★ 纯正铁路上盖双线枢纽极速通达
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>【房源】高楼层优质采光单位余货稀缺，推售现场需尽早锁定心仪朝向</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
@@ -1865,13 +1940,16 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龙城区校网名校网 ｜ 现楼</t>
+          <t>★ 何文田加多利山老牌名门贵胄地脉
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约1115米(约13分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共14伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
@@ -1928,13 +2006,16 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 何文田胜利道核心地段精品现楼
+🚇【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约554米(约6分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共71伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
@@ -1991,13 +2072,16 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 窝打老道93号/太子道西交界传统豪宅核心
+🚇【轨交】步行约 12 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角東站约971米(约11分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共56伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L24" s="3" t="inlineStr">
@@ -2054,13 +2138,16 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 加多利山与太子道西传统豪宅腹地
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁宋皇臺站约1045米(约12分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共45伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁宋皇臺站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
@@ -2117,13 +2204,16 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区三面临海极佳水岸占位
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
@@ -2180,13 +2270,16 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区三面临海极佳水岸占位
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
@@ -2243,18 +2336,22 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德城中心现楼发售即买即住即收租
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 9 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>步行约 5-6 分钟直达港铁启德站（屯马线），两站即达钻石山/宋皇台，畅达全港</t>
         </is>
       </c>
     </row>
@@ -2306,13 +2403,16 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道公园前排临海游艇景观
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
@@ -2369,13 +2469,16 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道公园前排临海游艇景观
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
@@ -2432,18 +2535,22 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德城中心前排紧邻启德河与港铁站
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>步行约 6-8 分钟直达港铁启德站（屯马线），立体路网贯穿港九</t>
         </is>
       </c>
     </row>
@@ -2495,18 +2602,22 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德城中心前排紧邻启德河与港铁站
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>步行约 6-8 分钟直达港铁启德站（屯马线），立体路网贯穿港九</t>
         </is>
       </c>
     </row>
@@ -2558,18 +2669,22 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德城中心前排紧邻启德河与港铁站
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>步行约 6-8 分钟直达港铁启德站（屯马线），立体路网贯穿港九</t>
         </is>
       </c>
     </row>
@@ -2621,18 +2736,22 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德城中心前排与双重视觉地标
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>步行约 5-7 分钟直达港铁启德站（屯马线），快速连通中环金钟及九龙东双CBD核心</t>
         </is>
       </c>
     </row>
@@ -2684,18 +2803,21 @@
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德城中心前排与双重视觉地标
+🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>步行约 5-7 分钟直达港铁启德站（屯马线），快速连通中环金钟及九龙东双CBD核心</t>
         </is>
       </c>
     </row>
@@ -2747,18 +2869,22 @@
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德城中心前排与双重视觉地标
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>步行约 5-7 分钟直达港铁启德站（屯马线），快速连通中环金钟及九龙东双CBD核心</t>
         </is>
       </c>
     </row>
@@ -2810,13 +2936,16 @@
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龙城区校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区核心海滨大型旗舰热销盘
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L37" s="3" t="inlineStr">
@@ -2873,13 +3002,16 @@
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龙城区校网名校网 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 启德跑道区核心海滨大型旗舰热销盘
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
@@ -2936,13 +3068,16 @@
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区龙头前排绝对一线临海地王
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
@@ -2999,18 +3134,22 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 紧邻港铁啟德站高效通勤</t>
+          <t>★ 启德唯一全天候无缝直达地铁新盘
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>港铁启德站无缝上盖核心枢纽，地下街直通车站及超甲级商厦AIRSIDE/双子汇；自驾经中九龙干线极速通达全港</t>
         </is>
       </c>
     </row>
@@ -3062,18 +3201,22 @@
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 港铁啟德站上盖/极速步行直达</t>
+          <t>★ 启德唯一全天候无缝直达地铁新盘
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>港铁启德站无缝上盖核心枢纽，地下街直通车站及超甲级商厦AIRSIDE/双子汇；自驾经中九龙干线极速通达全港</t>
         </is>
       </c>
     </row>
@@ -3125,13 +3268,16 @@
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区最前排半岛位龙头地王
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
@@ -3188,13 +3334,16 @@
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区最前排半岛位龙头地王
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr">
@@ -3251,13 +3400,16 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区最前排半岛位龙头地王
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr">
@@ -3314,13 +3466,16 @@
       </c>
       <c r="J45" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区三面环海绝佳占位
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
@@ -3377,13 +3532,16 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区三面环海绝佳占位
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
@@ -3440,13 +3598,16 @@
       </c>
       <c r="J47" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区三面环海绝佳占位
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
@@ -3503,13 +3664,16 @@
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区一线临海龙头
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr">
@@ -3566,13 +3730,16 @@
       </c>
       <c r="J49" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区首发大型地标住宅承丰道21号
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
@@ -3629,13 +3796,16 @@
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区核心承丰里2号双子地标
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L50" s="3" t="inlineStr">
@@ -3692,13 +3862,16 @@
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区前排龙头一线临海大宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L51" s="3" t="inlineStr">
@@ -3755,13 +3928,16 @@
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区前排龙头一线临海大宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
@@ -3818,13 +3994,16 @@
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 启德跑道区前排龙头一线临海大宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
@@ -3881,13 +4060,16 @@
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>港铁佐敦站上盖/极速步行直达 ｜ 现楼</t>
+          <t>★ 九龙佐敦德成街2号闹中取静绝佳地段
+🚇【轨交】步行约 2 分钟即达港铁佐敦站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合美丽华广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为31校网 / 油尖旺区校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共172伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L54" s="3" t="inlineStr">
@@ -3944,13 +4126,16 @@
       </c>
       <c r="J55" s="3" t="inlineStr">
         <is>
-          <t>乐风集团精工品质保障</t>
+          <t>★ 九龙繁华腹地界限街交通枢纽
+🚇【轨交】步行约 10 分钟即达港铁深水埗站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合西九龙中心等大型地标商圈
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁深水埗站约836米(约10分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为32校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L55" s="3" t="inlineStr">
@@ -4007,13 +4192,16 @@
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁太子站高效通勤 ｜ 乐风集团精工品质保障</t>
+          <t>★ 太子道西核心地脉步入双铁立体枢纽
+🚇【轨交】步行约 4 分钟即达港铁太子站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为32校网 / 油尖旺区校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共139伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L56" s="3" t="inlineStr">
@@ -4070,13 +4258,16 @@
       </c>
       <c r="J57" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 恒基兆业精工品质保障</t>
+          <t>★ 西九龙核心大角咀大型艺文商业街区
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁奧運站约909米(约10分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为32校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L57" s="3" t="inlineStr">
@@ -4133,13 +4324,16 @@
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 恒基兆业精工品质保障</t>
+          <t>★ 西九龙核心大角咀大型艺文商业街区
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁奧運站约909米(约10分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为32校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L58" s="3" t="inlineStr">
@@ -4196,13 +4390,16 @@
       </c>
       <c r="J59" s="3" t="inlineStr">
         <is>
-          <t>建灏地产 / 市建局精工品质保障</t>
+          <t>★ 西九龙大角咀核心生活圈交通极速通达
+🚇【轨交】步行约 10 分钟即达港铁旺角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁旺角站约819米(约9分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为32校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -4259,13 +4456,16 @@
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>东立地产精工品质保障</t>
+          <t>★ 九龙油麻地核心商圈全新精品住宅
+🚇【轨交】步行约 6 分钟即达港铁油麻地站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合朗豪坊等大型地标商圈</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为31校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共84伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L60" s="3" t="inlineStr">
@@ -4322,13 +4522,16 @@
       </c>
       <c r="J61" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 世茂集团精工品质保障</t>
+          <t>★ 九龙半山延坪道依山临海豪宅新地标
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁長沙灣站约2071米(约24分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🚇【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr">
@@ -4385,13 +4588,16 @@
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 新世界发展精工品质保障</t>
+          <t>★ 九龙塘又一村低密传世尊贵名邸
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站约1019米(约12分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L62" s="3" t="inlineStr">
@@ -4448,13 +4654,16 @@
       </c>
       <c r="J63" s="3" t="inlineStr">
         <is>
-          <t>恒基兆业精工品质保障</t>
+          <t>★ 红磡核心三轨枢纽立体交通网络
+🚇【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁何文田站约550米(约6分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L63" s="3" t="inlineStr">
@@ -4511,13 +4720,16 @@
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁何文田站高效通勤 ｜ 现楼</t>
+          <t>★ 九龙核心百万呎巨无霸都会重建
+🚇【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共324伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L64" s="3" t="inlineStr">
@@ -4574,13 +4786,16 @@
       </c>
       <c r="J65" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁何文田站高效通勤 ｜ 现楼</t>
+          <t>★ 九龙核心百万呎巨无霸都会重建
+🚇【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共280伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L65" s="3" t="inlineStr">
@@ -4637,13 +4852,16 @@
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>TKS LTD.精工品质保障</t>
+          <t>★ 九龙土瓜湾高山道公园旁清幽地段
+🚇【轨交】步行约 6 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共83伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L66" s="3" t="inlineStr">
@@ -4700,13 +4918,16 @@
       </c>
       <c r="J67" s="3" t="inlineStr">
         <is>
-          <t>恒基兆业 / 希慎兴业 / 帝国集团精工品质保障</t>
+          <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
+🚇【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约724米(约8分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L67" s="3" t="inlineStr">
@@ -4763,13 +4984,16 @@
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>恒基兆业 / 希慎兴业 / 帝国集团精工品质保障</t>
+          <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
+🚇【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约724米(约8分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L68" s="3" t="inlineStr">
@@ -4826,13 +5050,16 @@
       </c>
       <c r="J69" s="3" t="inlineStr">
         <is>
-          <t>恒基兆业 / 希慎兴业 / 帝国集团精工品质保障</t>
+          <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
+🚇【轨交】步行约 8 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约648米(约7分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L69" s="3" t="inlineStr">
@@ -4889,13 +5116,16 @@
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>恒基兆业 / 希慎兴业 / 帝国集团精工品质保障</t>
+          <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
+🚇【轨交】步行约 7 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站约598米(约7分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L70" s="3" t="inlineStr">
@@ -4952,13 +5182,16 @@
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>恒基兆业精工品质保障</t>
+          <t>★ 红磡核心枢纽珍罕999年期地契
+🚇【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁何文田站约599米(约7分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L71" s="3" t="inlineStr">
@@ -5015,13 +5248,16 @@
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>华润置地精工品质保障</t>
+          <t>★ 西南九龙绝版巨无霸大型发展区
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 10 分钟即达港铁荔枝角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁荔枝角站约874米(约10分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L72" s="3" t="inlineStr">
@@ -5078,18 +5314,21 @@
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 新鸿基地产 / 港铁精工品质保障</t>
+          <t>★ 港铁南昌站纯正铁路上盖双线枢纽
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁南昌站正上盖 / 直通（基座 V Walk 直通南昌站双铁枢纽）
+🛍️【商业】基座直连近 30 万呎 V Walk 大型综合商场
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁南昌站约571米(约6分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L73" s="3" t="inlineStr">
         <is>
-          <t>步行约 571米 (6分钟) 直达港铁南昌站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁南昌站正上盖物业（东涌线与屯马线双线交汇），一站直达西九龙高铁站及香港站（中环），极速贯通全港核心</t>
         </is>
       </c>
     </row>
@@ -5141,13 +5380,16 @@
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 会德丰 / 信和置业 / 嘉华国际 / 世茂 / 爪哇集团精工品质保障</t>
+          <t>★ 西南九龙绝版一线临海地王现楼
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁南昌站约1374米(约16分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为40校网 / 深水埗区校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🚇【交通】步行至最近港铁南昌站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L74" s="3" t="inlineStr">
@@ -5204,13 +5446,16 @@
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖41校网 / 九龍城校网名校网 ｜ 紧邻港铁宋皇臺站高效通勤</t>
+          <t>★ 九龙城宋皇台站步行约4-5分钟
+🚇【轨交】步行约 5 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>【社区】单幢式精致大厦(共313伙)，内部公用绿化及大型会所设施相对小巧 ；
-【交付】属预售楼花阶段(2025年入伙)，需等待工程竣工后交付</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L75" s="3" t="inlineStr">
@@ -5267,12 +5512,16 @@
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 紧邻港铁土瓜灣站高效通勤</t>
+          <t>★ 九龙土瓜湾核心大型重建标杆住区
+🚇【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>【交付】属预售楼花阶段(2027年入伙)，需等待工程竣工后交付</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L76" s="3" t="inlineStr">
@@ -5329,12 +5578,16 @@
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 紧邻港铁土瓜灣站高效通勤</t>
+          <t>★ 九龙土瓜湾核心大型重建标杆住区
+🚇【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>【交付】属预售楼花阶段(2027年入伙)，需等待工程竣工后交付</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L77" s="3" t="inlineStr">
@@ -5391,13 +5644,16 @@
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖41校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 九龙城联合道18号核心成熟板块
+🚇【轨交】步行约 7 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁宋皇臺站约559米(约6分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共92伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L78" s="3" t="inlineStr">
@@ -5454,13 +5710,16 @@
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>港铁炮台山站上盖/极速步行直达 ｜ 现楼</t>
+          <t>★ 港岛东核心北角英皇道绝佳占位
+🚇【轨交】步行约 3 分钟即达港铁炮台山站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为14校网 / 東區校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共251伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L79" s="3" t="inlineStr">
@@ -5517,13 +5776,16 @@
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>港铁北角站上盖/极速步行直达 ｜ 现楼</t>
+          <t>★ 港岛北角核心步行1-2分钟达北角站
+🚇【轨交】步行约 2 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为14校网 / 東區校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共281伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L80" s="3" t="inlineStr">
@@ -5580,12 +5842,16 @@
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 港铁天后站上盖/极速步行直达</t>
+          <t>★ 港岛核心天后站步行约3分钟
+🚇【轨交】步行约 3 分钟即达港铁天后站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>【社区】单幢式精致大厦(共74伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L81" s="3" t="inlineStr">
@@ -5642,13 +5908,16 @@
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 新世界 / 培新集团精工品质保障</t>
+          <t>★ 港岛东北角继园街大型旗舰园林私邸
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 8 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁北角站约661米(约7分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为14校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L82" s="3" t="inlineStr">
@@ -5705,12 +5974,16 @@
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁北角站高效通勤 ｜ 现楼</t>
+          <t>★ 港岛东一线临海绝版地王
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 5 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为14校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L83" s="3" t="inlineStr">
@@ -5767,12 +6040,16 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁北角站高效通勤 ｜ 现楼</t>
+          <t>★ 港岛东一线临海绝版地王
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 4 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为14校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L84" s="3" t="inlineStr">
@@ -5829,12 +6106,16 @@
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>港铁北角站上盖/极速步行直达 ｜ 现楼</t>
+          <t>★ 港岛东一线临海绝版地王
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 3 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为14校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L85" s="3" t="inlineStr">
@@ -5891,13 +6172,16 @@
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 中环半山己连拿利3号核心绝版地段
+🚇【轨交】步行约 9 分钟即达港铁中環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁中環站约734米(约8分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共99伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L86" s="3" t="inlineStr">
@@ -5954,12 +6238,16 @@
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 现楼</t>
+          <t>★ 东半山司徒拔道18号低密显赫豪宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁灣仔站约1708米(约20分钟)，建议接驳小巴至地铁</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L87" s="3" t="inlineStr">
@@ -6016,13 +6304,16 @@
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 现楼</t>
+          <t>★ 东半山司徒拔道18号低密显赫豪宅
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁灣仔站约1708米(约20分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共19伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L88" s="3" t="inlineStr">
@@ -6079,12 +6370,16 @@
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 中半山波老道21号香港顶奢豪宅标杆
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁金鐘站约1709米(约20分钟)，建议接驳小巴至地铁</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L89" s="3" t="inlineStr">
@@ -6141,13 +6436,16 @@
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 薄扶林道138号独立洋房顶奢地标
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁香港大學站约1152米(约13分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共7伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L90" s="3" t="inlineStr">
@@ -6204,13 +6502,16 @@
       </c>
       <c r="J91" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 港岛中环核心半山坚道黄金地段
+🚇【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约891米(约10分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共85伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L91" s="3" t="inlineStr">
@@ -6267,12 +6568,16 @@
       </c>
       <c r="J92" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 港岛西半山旭龢道42号显赫巅峰地段
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁香港大學站约1021米(约12分钟)，建议接驳小巴至地铁</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L92" s="3" t="inlineStr">
@@ -6329,13 +6634,16 @@
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 地段稀缺
+🚇【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约947米(约11分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共106伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L93" s="3" t="inlineStr">
@@ -6392,13 +6700,16 @@
       </c>
       <c r="J94" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 地段稀缺
+🚇【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约947米(约11分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共66伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L94" s="3" t="inlineStr">
@@ -6455,13 +6766,16 @@
       </c>
       <c r="J95" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 西半山宝珊道23号极低密16席传世大宅
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁香港大學站约1241米(约14分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共16伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L95" s="3" t="inlineStr">
@@ -6518,13 +6832,16 @@
       </c>
       <c r="J96" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 港岛西半山罗便臣道23号传统名门腹地
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约1146米(约13分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共90伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L96" s="3" t="inlineStr">
@@ -6581,12 +6898,16 @@
       </c>
       <c r="J97" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 中半山波老道21号传世顶奢大宅第2期
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁金鐘站约1764米(约21分钟)，建议接驳小巴至地铁</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L97" s="3" t="inlineStr">
@@ -6643,12 +6964,17 @@
       </c>
       <c r="J98" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 港岛西半山罗便臣道80号经典名牌豪宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 8 分钟即达港铁西營盤站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁西營盤站约650米(约7分钟)，建议接驳小巴至地铁</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L98" s="3" t="inlineStr">
@@ -6705,12 +7031,16 @@
       </c>
       <c r="J99" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 港铁堅尼地城站上盖/极速步行直达</t>
+          <t>★ 港岛西核心枢纽与极速通勤
+🚇【轨交】步行约 3 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K99" s="3" t="inlineStr">
         <is>
-          <t>【社区】单幢式精致大厦(共341伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L99" s="3" t="inlineStr">
@@ -6767,13 +7097,16 @@
       </c>
       <c r="J100" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西区校网名校网 ｜ 港铁堅尼地城站上盖/极速步行直达</t>
+          <t>★ 港岛西黄金地段步达坚尼地城站约2分钟
+🚇【轨交】步行约 2 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K100" s="3" t="inlineStr">
         <is>
-          <t>【社区】单幢式精致大厦(共173伙)，内部公用绿化及大型会所设施相对小巧 ；
-【交付】属预售楼花阶段(2025年入伙)，需等待工程竣工后交付</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L100" s="3" t="inlineStr">
@@ -6830,12 +7163,16 @@
       </c>
       <c r="J101" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 紧邻港铁堅尼地城站高效通勤</t>
+          <t>★ 港岛西坚尼地城临海一线视野
+🚇【轨交】步行约 5 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K101" s="3" t="inlineStr">
         <is>
-          <t>【社区】单幢式精致大厦(共125伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L101" s="3" t="inlineStr">
@@ -6892,13 +7229,16 @@
       </c>
       <c r="J102" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 港岛南区大潭白笔山道一线纯独立海景洋房
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K102" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L102" s="3" t="inlineStr">
@@ -6955,13 +7295,16 @@
       </c>
       <c r="J103" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 英皇国际 / 中渝置地 / 明发集团 / 尚家生活精工品质保障</t>
+          <t>★ 港岛南区传统顶级显赫富豪圈
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K103" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L103" s="3" t="inlineStr">
@@ -7018,13 +7361,16 @@
       </c>
       <c r="J104" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 新鸿基地产精工品质保障</t>
+          <t>★ 浅水湾道3号港岛南区顶级老牌超级豪宅
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K104" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L104" s="3" t="inlineStr">
@@ -7081,13 +7427,16 @@
       </c>
       <c r="J105" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 新鸿基地产精工品质保障</t>
+          <t>★ 港岛南区寿臣山顶级独立洋房群
+🚇【轨交】步行约 12 分钟即达港铁海洋公園站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K105" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南区校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L105" s="3" t="inlineStr">
@@ -7144,13 +7493,16 @@
       </c>
       <c r="J106" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 浅水湾道108号极度珍罕独立海景洋房
+🛍️【商业】邻近/周边1.5km聚合The Pulse等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K106" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南区校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L106" s="3" t="inlineStr">
@@ -7207,13 +7559,16 @@
       </c>
       <c r="J107" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 港岛南区深水湾径超级隐秘纯豪宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K107" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L107" s="3" t="inlineStr">
@@ -7270,13 +7625,16 @@
       </c>
       <c r="J108" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 现楼</t>
+          <t>★ 香港山顶聂歌信山道亚洲顶奢楼王地标
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K108" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【配套】纯住宅静谧地脉自身底商精简，大型商业采买依赖短途车程接驳</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L108" s="3" t="inlineStr">
@@ -7333,13 +7691,16 @@
       </c>
       <c r="J109" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 现楼</t>
+          <t>★ 香港山顶聂歌信山道亚洲顶奢楼王地标
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K109" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【配套】纯住宅静谧地脉自身底商精简，大型商业采买依赖短途车程接驳</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L109" s="3" t="inlineStr">
@@ -7396,13 +7757,16 @@
       </c>
       <c r="J110" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西区校网名校网 ｜ 现楼</t>
+          <t>★ 香港山顶加列山道12号巅峰独立洋房群
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K110" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【配套】纯住宅静谧地脉自身底商精简，大型商业采买依赖短途车程接驳</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L110" s="3" t="inlineStr">
@@ -7459,13 +7823,16 @@
       </c>
       <c r="J111" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西区校网名校网 ｜ 现楼</t>
+          <t>★ 香港山顶宾吉道3号太古地产传世洋房
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K111" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【配套】纯住宅静谧地脉自身底商精简，大型商业采买依赖短途车程接驳</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L111" s="3" t="inlineStr">
@@ -7522,13 +7889,16 @@
       </c>
       <c r="J112" s="3" t="inlineStr">
         <is>
-          <t>一线维港海滨/开阔海湾稀缺视野 ｜ 太古地产精工品质保障</t>
+          <t>★ 太古地产港岛东柴湾罕见大型综合体
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K112" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁柴灣站约945米(约11分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为16校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L112" s="3" t="inlineStr">
@@ -7585,12 +7955,16 @@
       </c>
       <c r="J113" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 现楼</t>
+          <t>★ 渣甸山30年唯一罕见分层新盘
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K113" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁天后站约1809米(约21分钟)，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L113" s="3" t="inlineStr">
@@ -7647,13 +8021,16 @@
       </c>
       <c r="J114" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 现楼</t>
+          <t>★ 港岛湾仔活道15号核心成熟地段
+🚇【轨交】步行约 9 分钟即达港铁灣仔站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合时代广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K114" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁灣仔站约715米(约8分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共167伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L114" s="3" t="inlineStr">
@@ -7710,13 +8087,16 @@
       </c>
       <c r="J115" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁西灣河站高效通勤 ｜ 现楼</t>
+          <t>★ 港岛东核心西湾河站步行约4分钟
+🚇【轨交】步行约 4 分钟即达港铁西灣河站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K115" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为16校网 / 東區校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共57伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L115" s="3" t="inlineStr">
@@ -7773,13 +8153,16 @@
       </c>
       <c r="J116" s="3" t="inlineStr">
         <is>
-          <t>港铁筲箕灣站上盖/极速步行直达 ｜ 现楼</t>
+          <t>★ 港岛东筲箕湾站步行约3分钟
+🚇【轨交】步行约 3 分钟即达港铁筲箕灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K116" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为16校网 / 東區校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共156伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L116" s="3" t="inlineStr">
@@ -7836,13 +8219,16 @@
       </c>
       <c r="J117" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 协成行精工品质保障</t>
+          <t>★ 港岛东核心筲箕湾东大街23号成熟商圈
+🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K117" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁筲箕灣站约1073米(约12分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为16校网 / 东区校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁筲箕灣站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L117" s="3" t="inlineStr">
@@ -7899,13 +8285,16 @@
       </c>
       <c r="J118" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 华懋集团精工品质保障</t>
+          <t>★ 薄扶林域多利道301号全海景现楼
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🛍️【商业】邻近/周边1.5km聚合数码港商场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K118" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁堅尼地城站约1541米(约18分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🚇【交通】步行至最近港铁堅尼地城站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L118" s="3" t="inlineStr">
@@ -7962,13 +8351,16 @@
       </c>
       <c r="J119" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 港铁西營盤站上盖/极速步行直达</t>
+          <t>★ 港岛西营盘核心枢纽极速通达
+🚇【轨交】步行约 3 分钟即达港铁西營盤站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈</t>
         </is>
       </c>
       <c r="K119" s="3" t="inlineStr">
         <is>
-          <t>【社区】单幢式精致大厦(共105伙)，内部公用绿化及大型会所设施相对小巧 ；
-【交付】属预售楼花阶段(即将发售)，需等待工程竣工后交付</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L119" s="3" t="inlineStr">
@@ -8025,13 +8417,16 @@
       </c>
       <c r="J120" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖11校网 / 中西區校网名校网 ｜ 现楼</t>
+          <t>★ 上环苏豪艺术区极低密顶奢私邸
+🚇【轨交】步行约 7 分钟即达港铁上環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K120" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁上環站约555米(约6分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共13伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L120" s="3" t="inlineStr">
@@ -8088,13 +8483,16 @@
       </c>
       <c r="J121" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 新鸿基地产精工品质保障</t>
+          <t>★ 港岛南区赤柱村道纯正低密滨海豪宅
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K121" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L121" s="3" t="inlineStr">
@@ -8151,13 +8549,16 @@
       </c>
       <c r="J122" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 建灏地产精工品质保障</t>
+          <t>★ 港岛南区赤柱黄麻角道纯海景洋房及大宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K122" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L122" s="3" t="inlineStr">
@@ -8214,13 +8615,16 @@
       </c>
       <c r="J123" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 东立地产精工品质保障</t>
+          <t>★ 港岛南区寿臣山道西稀缺纯独立洋房
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K123" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L123" s="3" t="inlineStr">
@@ -8277,13 +8681,16 @@
       </c>
       <c r="J124" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 港岛南区舂磡角海天径绝版5席独立大宅
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K124" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L124" s="3" t="inlineStr">
@@ -8340,13 +8747,16 @@
       </c>
       <c r="J125" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 培新集团精工品质保障</t>
+          <t>★ 赤柱半山环角道隐秘低密独栋纯墅区
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K125" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南区校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L125" s="3" t="inlineStr">
@@ -8403,13 +8813,16 @@
       </c>
       <c r="J126" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 湾仔区校网名校网 ｜ 现楼</t>
+          <t>★ 东半山大坑道339号传统显赫地段
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K126" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【配套】纯住宅静谧地脉自身底商精简，大型商业采买依赖短途车程接驳</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L126" s="3" t="inlineStr">
@@ -8466,13 +8879,16 @@
       </c>
       <c r="J127" s="3" t="inlineStr">
         <is>
-          <t>港铁黃竹坑站上盖/极速步行直达 ｜ 长江实业 / 港铁精工品质保障</t>
+          <t>★ 港铁黄竹坑站上盖专属电梯直达
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K127" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校 ；
-【交付】属预售楼花阶段(2025年入伙)，需等待工程竣工后交付</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L127" s="3" t="inlineStr">
@@ -8529,13 +8945,16 @@
       </c>
       <c r="J128" s="3" t="inlineStr">
         <is>
-          <t>港铁黃竹坑站上盖/极速步行直达 ｜ 长江实业 / 港铁精工品质保障</t>
+          <t>★ 港铁黄竹坑站上盖专属电梯直达
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K128" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校 ；
-【交付】属预售楼花阶段(2025年入伙)，需等待工程竣工后交付</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L128" s="3" t="inlineStr">
@@ -8592,12 +9011,16 @@
       </c>
       <c r="J129" s="3" t="inlineStr">
         <is>
-          <t>港铁黃竹坑站上盖/极速步行直达 ｜ 现楼</t>
+          <t>★ 港岛30年唯一新房地铁上盖
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K129" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L129" s="3" t="inlineStr">
@@ -8654,12 +9077,16 @@
       </c>
       <c r="J130" s="3" t="inlineStr">
         <is>
-          <t>港铁黃竹坑站上盖/极速步行直达 ｜ 现楼</t>
+          <t>★ 港岛30年唯一新房地铁上盖
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K130" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L130" s="3" t="inlineStr">
@@ -8716,13 +9143,16 @@
       </c>
       <c r="J131" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁利東站高效通勤 ｜ 现楼</t>
+          <t>★ 港岛南区鸭脷洲海旁水岸生活圈
+🚇【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K131" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共174伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L131" s="3" t="inlineStr">
@@ -8779,13 +9209,16 @@
       </c>
       <c r="J132" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 庄士机构精工品质保障</t>
+          <t>★ 港岛南区鸭脷洲平澜街滨海水岸新盘
+🚇【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K132" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共105伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L132" s="3" t="inlineStr">
@@ -8842,18 +9275,21 @@
       </c>
       <c r="J133" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 港铁黄竹坑站上盖港岛南岸第2期
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直连车站大堂）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K133" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁黃竹坑站约624米(约7分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L133" s="3" t="inlineStr">
         <is>
-          <t>步行约 624米 (7分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁黄竹坑站正上盖港岛南岸（南港岛线），两站直达金钟核心枢纽，商场THE SOUTHSIDE无缝直连</t>
         </is>
       </c>
     </row>
@@ -8905,12 +9341,16 @@
       </c>
       <c r="J134" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁黃竹坑站高效通勤 ｜ 现楼</t>
+          <t>★ 港铁黄竹坑站上盖港岛南岸首发旗舰项目
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座直连 THE SOUTHSIDE 商场与车站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K134" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L134" s="3" t="inlineStr">
@@ -8967,12 +9407,16 @@
       </c>
       <c r="J135" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁黃竹坑站高效通勤 ｜ 现楼</t>
+          <t>★ 港铁黄竹坑站纯正铁路上盖
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K135" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L135" s="3" t="inlineStr">
@@ -9029,12 +9473,16 @@
       </c>
       <c r="J136" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁黃竹坑站高效通勤 ｜ 现楼</t>
+          <t>★ 港铁黄竹坑站纯正铁路上盖
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K136" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L136" s="3" t="inlineStr">
@@ -9091,13 +9539,16 @@
       </c>
       <c r="J137" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁黃竹坑站高效通勤 ｜ 新世界 / 帝国集团 / 资本策略 / 丽新发展 / 港铁精工品质保障</t>
+          <t>★ 港铁黄竹坑站上盖港岛南岸第5期
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
         </is>
       </c>
       <c r="K137" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校 ；
-【交付】属预售楼花阶段(2026年入伙)，需等待工程竣工后交付</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L137" s="3" t="inlineStr">
@@ -9154,13 +9605,16 @@
       </c>
       <c r="J138" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 港岛南区鸭脷洲海旁道一线游艇海景
+🚇【轨交】步行约 11 分钟即达港铁利東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K138" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁利東站约892米(约10分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L138" s="3" t="inlineStr">
@@ -9217,13 +9671,16 @@
       </c>
       <c r="J139" s="3" t="inlineStr">
         <is>
-          <t>港铁利東站上盖/极速步行直达 ｜ 现楼</t>
+          <t>★ 港岛南区鸭脷洲大街步行约3分钟达利东站
+🚇【轨交】步行约 3 分钟即达港铁利東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K139" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共138伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L139" s="3" t="inlineStr">
@@ -9280,12 +9737,16 @@
       </c>
       <c r="J140" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁鰂魚涌站高效通勤 ｜ 现楼</t>
+          <t>★ 港岛东核心鲗鱼涌站步行约4分钟
+🚇【轨交】步行约 4 分钟即达港铁鰂魚涌站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K140" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为14校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L140" s="3" t="inlineStr">
@@ -9342,13 +9803,16 @@
       </c>
       <c r="J141" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 龙光集团 / 合景泰富精工品质保障</t>
+          <t>★ 港岛南区鸭脷洲一线临海现楼超级豪宅
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 7 分钟即达港铁海怡半島站（轨交通勤从容便捷）
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K141" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁海怡半島站约594米(约7分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L141" s="3" t="inlineStr">
@@ -9405,13 +9869,16 @@
       </c>
       <c r="J142" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 现楼</t>
+          <t>★ 跑马地桂芳街8号老牌名流核心区
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K142" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁銅鑼灣站约1891米(约22分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共156伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L142" s="3" t="inlineStr">
@@ -9468,13 +9935,16 @@
       </c>
       <c r="J143" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 现楼</t>
+          <t>★ 跑马地蓝塘道半山珍罕大型洋房群
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K143" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁銅鑼灣站约1824米(约21分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共18伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L143" s="3" t="inlineStr">
@@ -9531,18 +10001,21 @@
       </c>
       <c r="J144" s="3" t="inlineStr">
         <is>
-          <t>新世界 / 帝国集团 / 资本策略 / 丽新发展 / 港铁精工品质保障</t>
+          <t>★ 港铁黄竹坑站上盖港岛南岸第5期
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
         </is>
       </c>
       <c r="K144" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁黃竹坑站约598米(约7分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L144" s="3" t="inlineStr">
         <is>
-          <t>步行约 598米 (7分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁黄竹坑站正上盖港岛南岸（南港岛线），两站直达金钟核心枢纽，商场THE SOUTHSIDE无缝直连</t>
         </is>
       </c>
     </row>
@@ -9594,13 +10067,16 @@
       </c>
       <c r="J145" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龙城区校网名校网 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 启德跑道区承丰道16号海滨前排新地标
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
         </is>
       </c>
       <c r="K145" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L145" s="3" t="inlineStr">
@@ -9657,13 +10133,16 @@
       </c>
       <c r="J146" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龙城区校网名校网 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 启德跑道区承丰道16号海滨前排新地标
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
         </is>
       </c>
       <c r="K146" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处启德跑道区，日常需搭乘专线巴士约5-8分钟接驳至港铁启德站/宋皇台站 ；
-【配套】滨海商业街区处于逐步兑现期，现阶段大型商业依赖启德城中心AIRSIDE/双子汇</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L146" s="3" t="inlineStr">
@@ -9720,13 +10199,16 @@
       </c>
       <c r="J147" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁旺角東站高效通勤 ｜ 现楼</t>
+          <t>★ 旺角核心洗衣街地段步入太子及旺角东双铁
+🚇【轨交】步行约 5 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K147" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为32校网 / 油尖旺校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共52伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L147" s="3" t="inlineStr">
@@ -9783,13 +10265,16 @@
       </c>
       <c r="J148" s="3" t="inlineStr">
         <is>
-          <t>现楼 ｜ 会德丰 / 信和置业 / 嘉华国际 / 世茂 / 爪哇集团精工品质保障</t>
+          <t>★ 西南九龙绝版一线临海地王现楼
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K148" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁南昌站约1247米(约15分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为40校网 / 深水埗区校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🚇【交通】步行至最近港铁南昌站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L148" s="3" t="inlineStr">
@@ -9846,13 +10331,16 @@
       </c>
       <c r="J149" s="3" t="inlineStr">
         <is>
-          <t>信和 / 华懋集团 / 亚证地产精工品质保障</t>
+          <t>★ 港岛大潭白笔山道18号经典滨海独立洋房</t>
         </is>
       </c>
       <c r="K149" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L149" s="3" t="inlineStr">
@@ -9909,13 +10397,16 @@
       </c>
       <c r="J150" s="3" t="inlineStr">
         <is>
-          <t>信和 / 华懋集团 / 亚证地产精工品质保障</t>
+          <t>★ 港岛大潭白笔山道18号经典滨海独立洋房</t>
         </is>
       </c>
       <c r="K150" s="3" t="inlineStr">
         <is>
-          <t>【交通】纯自住低密地脉无就近港铁站，日常出行高度依赖私家车或专属车队 ；
-【校网】所属公立校网为18校网 / 南區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L150" s="3" t="inlineStr">
@@ -9972,12 +10463,16 @@
       </c>
       <c r="J151" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖34校网 / 九龍城校网名校网 ｜ 现楼</t>
+          <t>★ 何文田自由道传统静谧高尚住宅地脉
+🚇【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K151" s="3" t="inlineStr">
         <is>
-          <t>【社区】单幢式精致大厦(共91伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L151" s="3" t="inlineStr">
@@ -10034,13 +10529,16 @@
       </c>
       <c r="J152" s="3" t="inlineStr">
         <is>
-          <t>一线维港海滨/开阔海湾稀缺视野 ｜ 太古地产精工品质保障</t>
+          <t>★ 太古地产港岛东柴湾罕见大型综合体
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈</t>
         </is>
       </c>
       <c r="K152" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁柴灣站约945米(约11分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为16校网 / 東區校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L152" s="3" t="inlineStr">
@@ -10097,13 +10595,16 @@
       </c>
       <c r="J153" s="3" t="inlineStr">
         <is>
-          <t>华润置地精工品质保障</t>
+          <t>★ 西南九龙绝版巨无霸大型发展区
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】步行约 10 分钟即达港铁長沙灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
         </is>
       </c>
       <c r="K153" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁長沙灣站约817米(约10分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为40校网 / 深水埗校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L153" s="3" t="inlineStr">
@@ -10160,13 +10661,16 @@
       </c>
       <c r="J154" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁何文田站高效通勤 ｜ 恒基兆业精工品质保障</t>
+          <t>★ 九龙核心百万呎巨无霸都会重建
+🚇【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
         </is>
       </c>
       <c r="K154" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为35校网 / 九龍城校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共263伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L154" s="3" t="inlineStr">
@@ -10223,13 +10727,16 @@
       </c>
       <c r="J155" s="3" t="inlineStr">
         <is>
-          <t>全港顶尖12校网 / 灣仔校网名校网 ｜ 现楼</t>
+          <t>★ 港岛东半山肇辉台6号极度低密传世私邸
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利东街等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K155" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁灣仔站约1065米(约13分钟)，建议接驳小巴至地铁 ；
-【社区】单幢式精致大厦(共24伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L155" s="3" t="inlineStr">
@@ -10286,13 +10793,16 @@
       </c>
       <c r="J156" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁康城站高效通勤 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 港铁康城站临海前排一线开扬全海景
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
+🛍️【商业】连桥直达 The LOHAS 康城地标级商场</t>
         </is>
       </c>
       <c r="K156" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为95校网 / 西貢校网，重视升学建议结合片区优质私立或国际学校 ；
-【交付】属预售楼花阶段(2027年入伙)，需等待工程竣工后交付</t>
+          <t>🎓【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L156" s="3" t="inlineStr">
@@ -10349,13 +10859,16 @@
       </c>
       <c r="J157" s="3" t="inlineStr">
         <is>
-          <t>港铁康城站上盖/极速步行直达 ｜ 一线维港海滨/开阔海湾稀缺视野</t>
+          <t>★ 港铁康城站临海前排一线开扬全海景
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🚇【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
+🛍️【商业】连桥直达 The LOHAS 康城地标级商场</t>
         </is>
       </c>
       <c r="K157" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为95校网 / 西貢校网，重视升学建议结合片区优质私立或国际学校 ；
-【交付】属预售楼花阶段(2027年入伙)，需等待工程竣工后交付</t>
+          <t>🎓【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L157" s="3" t="inlineStr">
@@ -10412,13 +10925,16 @@
       </c>
       <c r="J158" s="3" t="inlineStr">
         <is>
-          <t>紧邻港铁炮台山站高效通勤 ｜ 周大福精工品质保障</t>
+          <t>★ 北角核心繁华腹地与成熟商圈
+🚇【轨交】步行约 6 分钟即达港铁炮台山站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈</t>
         </is>
       </c>
       <c r="K158" s="3" t="inlineStr">
         <is>
-          <t>【校网】所属公立校网为14校网 / 东区校网，重视升学建议结合片区优质私立或国际学校 ；
-【社区】单幢式精致大厦(共194伙)，内部公用绿化及大型会所设施相对小巧</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L158" s="3" t="inlineStr">
@@ -10475,13 +10991,16 @@
       </c>
       <c r="J159" s="3" t="inlineStr">
         <is>
-          <t>恒基兆业精工品质保障</t>
+          <t>★ 恒基西九龙市区更新全新力作
+🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈</t>
         </is>
       </c>
       <c r="K159" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁太子站约1028米(约12分钟)，建议接驳小巴至地铁 ；
-【校网】所属公立校网为32校网 / 油尖旺区校网，重视升学建议结合片区优质私立或国际学校</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】步行至最近港铁太子站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
+⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L159" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fix(export): remove redundant emojis 🚇, 🎓, 🛍️ in 5D tradeoff pills
</commit_message>
<xml_diff>
--- a/导出方案项目描述库.xlsx
+++ b/导出方案项目描述库.xlsx
@@ -618,14 +618,14 @@
         <is>
           <t>★ 九龙塘龙庭里8号超级豪宅巅峰之作
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
+          <t>【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
@@ -683,15 +683,15 @@
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>★ 九龙塘龙庭里8号超级豪宅巅峰之作
-🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -749,15 +749,15 @@
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>★ 九龙塘龙庭里8号超级豪宅巅峰之作
-🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -816,14 +816,14 @@
         <is>
           <t>★ 九龙塘广播道半山珍稀向南大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
+          <t>【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
@@ -881,15 +881,15 @@
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>★ 九龙塘喇沙利道32-38号喇沙小学正对面
-🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
@@ -948,14 +948,14 @@
         <is>
           <t>★ 九龙笔架山半山龙驹道超级豪宅巅峰
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
-🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
+【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
@@ -1014,14 +1014,14 @@
         <is>
           <t>★ 九龙站上盖香港地标级顶奢天际豪宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁九龙站正上盖 / 直通（直通圆方 ELEMENTS 与九龙站/柯士甸）
-🛍️【商业】基座直通圆方 ELEMENTS 超大型购物中心
+【轨交】港铁九龙站正上盖 / 直通（直通圆方 ELEMENTS 与九龙站/柯士甸）
+️【商业】基座直通圆方 ELEMENTS 超大型购物中心
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
@@ -1079,15 +1079,15 @@
       <c r="J9" s="3" t="inlineStr">
         <is>
           <t>★ 何文田窝打老道黄金名校地段
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
@@ -1145,9 +1145,9 @@
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>★ 太子道西核心地段新鸿基品质力作
-🚇【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1211,9 +1211,9 @@
       <c r="J11" s="3" t="inlineStr">
         <is>
           <t>★ 何文田自由道万科品质轻奢地标
-🚇【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1278,9 +1278,9 @@
         <is>
           <t>★ 何文田加多利山百年名门显赫地段
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1345,14 +1345,14 @@
         <is>
           <t>★ 何文田核心传统豪宅区现楼大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
+          <t>【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1410,15 +1410,15 @@
       <c r="J14" s="3" t="inlineStr">
         <is>
           <t>★ 太子道西266号传统豪宅名门腹地
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
@@ -1477,9 +1477,9 @@
         <is>
           <t>★ 何文田佛光街23号新鸿基巅峰豪宅标杆
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1543,9 +1543,9 @@
       <c r="J16" s="3" t="inlineStr">
         <is>
           <t>★ 九龙顶尖34名校网黄金护城河
-🚇【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1609,15 +1609,15 @@
       <c r="J17" s="3" t="inlineStr">
         <is>
           <t>★ 太子道西279号极低密名门大宅
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -1676,9 +1676,9 @@
         <is>
           <t>★ 港铁何文田站纯正铁路上盖绝版压轴大盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -1742,9 +1742,9 @@
         <is>
           <t>★ 港铁何文田站纯正铁路上盖绝版压轴大盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -1808,9 +1808,9 @@
         <is>
           <t>★ 纯正铁路上盖双线枢纽极速通达
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
@@ -1875,9 +1875,9 @@
         <is>
           <t>★ 纯正铁路上盖双线枢纽极速通达
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1941,15 +1941,15 @@
       <c r="J22" s="3" t="inlineStr">
         <is>
           <t>★ 何文田加多利山老牌名门贵胄地脉
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
@@ -2007,9 +2007,9 @@
       <c r="J23" s="3" t="inlineStr">
         <is>
           <t>★ 何文田胜利道核心地段精品现楼
-🚇【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2073,9 +2073,9 @@
       <c r="J24" s="3" t="inlineStr">
         <is>
           <t>★ 窝打老道93号/太子道西交界传统豪宅核心
-🚇【轨交】步行约 12 分钟即达港铁旺角東站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【轨交】步行约 12 分钟即达港铁旺角東站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2139,15 +2139,15 @@
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>★ 加多利山与太子道西传统豪宅腹地
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁宋皇臺站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁宋皇臺站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
@@ -2206,14 +2206,14 @@
         <is>
           <t>★ 启德跑道区三面临海极佳水岸占位
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
@@ -2272,14 +2272,14 @@
         <is>
           <t>★ 启德跑道区三面临海极佳水岸占位
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
@@ -2338,9 +2338,9 @@
         <is>
           <t>★ 启德城中心现楼发售即买即住即收租
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 9 分钟即达港铁啟德站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈
+【轨交】步行约 9 分钟即达港铁啟德站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2405,14 +2405,14 @@
         <is>
           <t>★ 启德跑道公园前排临海游艇景观
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
@@ -2471,14 +2471,14 @@
         <is>
           <t>★ 启德跑道公园前排临海游艇景观
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
@@ -2537,9 +2537,9 @@
         <is>
           <t>★ 启德城中心前排紧邻启德河与港铁站
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2604,9 +2604,9 @@
         <is>
           <t>★ 启德城中心前排紧邻启德河与港铁站
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2671,9 +2671,9 @@
         <is>
           <t>★ 启德城中心前排紧邻启德河与港铁站
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2738,9 +2738,9 @@
         <is>
           <t>★ 启德城中心前排与双重视觉地标
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2804,9 +2804,9 @@
       <c r="J35" s="3" t="inlineStr">
         <is>
           <t>★ 启德城中心前排与双重视觉地标
-🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2871,9 +2871,9 @@
         <is>
           <t>★ 启德城中心前排与双重视觉地标
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2938,14 +2938,14 @@
         <is>
           <t>★ 启德跑道区核心海滨大型旗舰热销盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L37" s="3" t="inlineStr">
@@ -3004,14 +3004,14 @@
         <is>
           <t>★ 启德跑道区核心海滨大型旗舰热销盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
@@ -3070,14 +3070,14 @@
         <is>
           <t>★ 启德跑道区龙头前排绝对一线临海地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
@@ -3136,9 +3136,9 @@
         <is>
           <t>★ 启德唯一全天候无缝直达地铁新盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
+【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -3203,9 +3203,9 @@
         <is>
           <t>★ 启德唯一全天候无缝直达地铁新盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
+【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -3270,14 +3270,14 @@
         <is>
           <t>★ 启德跑道区最前排半岛位龙头地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
@@ -3335,15 +3335,15 @@
       <c r="J43" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区最前排半岛位龙头地王
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr">
@@ -3402,14 +3402,14 @@
         <is>
           <t>★ 启德跑道区最前排半岛位龙头地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr">
@@ -3468,14 +3468,14 @@
         <is>
           <t>★ 启德跑道区三面环海绝佳占位
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
@@ -3534,14 +3534,14 @@
         <is>
           <t>★ 启德跑道区三面环海绝佳占位
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
@@ -3599,15 +3599,15 @@
       <c r="J47" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区三面环海绝佳占位
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
@@ -3666,14 +3666,14 @@
         <is>
           <t>★ 启德跑道区一线临海龙头
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr">
@@ -3731,15 +3731,15 @@
       <c r="J49" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区首发大型地标住宅承丰道21号
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
@@ -3798,14 +3798,14 @@
         <is>
           <t>★ 启德跑道区核心承丰里2号双子地标
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L50" s="3" t="inlineStr">
@@ -3864,14 +3864,14 @@
         <is>
           <t>★ 启德跑道区前排龙头一线临海大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L51" s="3" t="inlineStr">
@@ -3930,14 +3930,14 @@
         <is>
           <t>★ 启德跑道区前排龙头一线临海大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
@@ -3996,14 +3996,14 @@
         <is>
           <t>★ 启德跑道区前排龙头一线临海大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
@@ -4061,15 +4061,15 @@
       <c r="J54" s="3" t="inlineStr">
         <is>
           <t>★ 九龙佐敦德成街2号闹中取静绝佳地段
-🚇【轨交】步行约 2 分钟即达港铁佐敦站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合美丽华广场等大型地标商圈
+【轨交】步行约 2 分钟即达港铁佐敦站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合美丽华广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L54" s="3" t="inlineStr">
@@ -4127,15 +4127,15 @@
       <c r="J55" s="3" t="inlineStr">
         <is>
           <t>★ 九龙繁华腹地界限街交通枢纽
-🚇【轨交】步行约 10 分钟即达港铁深水埗站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合西九龙中心等大型地标商圈
+【轨交】步行约 10 分钟即达港铁深水埗站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合西九龙中心等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L55" s="3" t="inlineStr">
@@ -4193,14 +4193,14 @@
       <c r="J56" s="3" t="inlineStr">
         <is>
           <t>★ 太子道西核心地脉步入双铁立体枢纽
-🚇【轨交】步行约 4 分钟即达港铁太子站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈</t>
+【轨交】步行约 4 分钟即达港铁太子站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -4260,14 +4260,14 @@
         <is>
           <t>★ 西九龙核心大角咀大型艺文商业街区
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
+【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L57" s="3" t="inlineStr">
@@ -4326,14 +4326,14 @@
         <is>
           <t>★ 西九龙核心大角咀大型艺文商业街区
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
+【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L58" s="3" t="inlineStr">
@@ -4391,15 +4391,15 @@
       <c r="J59" s="3" t="inlineStr">
         <is>
           <t>★ 西九龙大角咀核心生活圈交通极速通达
-🚇【轨交】步行约 10 分钟即达港铁旺角站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
+【轨交】步行约 10 分钟即达港铁旺角站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -4457,14 +4457,14 @@
       <c r="J60" s="3" t="inlineStr">
         <is>
           <t>★ 九龙油麻地核心商圈全新精品住宅
-🚇【轨交】步行约 6 分钟即达港铁油麻地站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合朗豪坊等大型地标商圈</t>
+【轨交】步行约 6 分钟即达港铁油麻地站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合朗豪坊等大型地标商圈</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -4529,9 +4529,9 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
-🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
+【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr">
@@ -4589,15 +4589,15 @@
       <c r="J62" s="3" t="inlineStr">
         <is>
           <t>★ 九龙塘又一村低密传世尊贵名邸
-🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁
-🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁
+【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L62" s="3" t="inlineStr">
@@ -4655,15 +4655,15 @@
       <c r="J63" s="3" t="inlineStr">
         <is>
           <t>★ 红磡核心三轨枢纽立体交通网络
-🚇【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
+【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L63" s="3" t="inlineStr">
@@ -4721,15 +4721,15 @@
       <c r="J64" s="3" t="inlineStr">
         <is>
           <t>★ 九龙核心百万呎巨无霸都会重建
-🚇【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
+【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L64" s="3" t="inlineStr">
@@ -4787,15 +4787,15 @@
       <c r="J65" s="3" t="inlineStr">
         <is>
           <t>★ 九龙核心百万呎巨无霸都会重建
-🚇【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
+【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L65" s="3" t="inlineStr">
@@ -4853,15 +4853,15 @@
       <c r="J66" s="3" t="inlineStr">
         <is>
           <t>★ 九龙土瓜湾高山道公园旁清幽地段
-🚇【轨交】步行约 6 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+【轨交】步行约 6 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L66" s="3" t="inlineStr">
@@ -4919,14 +4919,14 @@
       <c r="J67" s="3" t="inlineStr">
         <is>
           <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
-🚇【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -4985,14 +4985,14 @@
       <c r="J68" s="3" t="inlineStr">
         <is>
           <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
-🚇【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
+【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -5051,14 +5051,14 @@
       <c r="J69" s="3" t="inlineStr">
         <is>
           <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
-🚇【轨交】步行约 8 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+【轨交】步行约 8 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -5117,14 +5117,14 @@
       <c r="J70" s="3" t="inlineStr">
         <is>
           <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
-🚇【轨交】步行约 7 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+【轨交】步行约 7 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -5183,14 +5183,14 @@
       <c r="J71" s="3" t="inlineStr">
         <is>
           <t>★ 红磡核心枢纽珍罕999年期地契
-🚇【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
+【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -5250,13 +5250,13 @@
         <is>
           <t>★ 西南九龙绝版巨无霸大型发展区
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 10 分钟即达港铁荔枝角站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
+【轨交】步行约 10 分钟即达港铁荔枝角站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
+          <t>【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -5316,14 +5316,14 @@
         <is>
           <t>★ 港铁南昌站纯正铁路上盖双线枢纽
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁南昌站正上盖 / 直通（基座 V Walk 直通南昌站双铁枢纽）
-🛍️【商业】基座直连近 30 万呎 V Walk 大型综合商场
+【轨交】港铁南昌站正上盖 / 直通（基座 V Walk 直通南昌站双铁枢纽）
+️【商业】基座直连近 30 万呎 V Walk 大型综合商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L73" s="3" t="inlineStr">
@@ -5382,14 +5382,14 @@
         <is>
           <t>★ 西南九龙绝版一线临海地王现楼
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
+️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】步行至最近港铁南昌站超12分钟，建议接驳小巴至地铁
-🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【交通】步行至最近港铁南昌站超12分钟，建议接驳小巴至地铁
+【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L74" s="3" t="inlineStr">
@@ -5447,9 +5447,9 @@
       <c r="J75" s="3" t="inlineStr">
         <is>
           <t>★ 九龙城宋皇台站步行约4-5分钟
-🚇【轨交】步行约 5 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
+【轨交】步行约 5 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
+【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
@@ -5513,9 +5513,9 @@
       <c r="J76" s="3" t="inlineStr">
         <is>
           <t>★ 九龙土瓜湾核心大型重建标杆住区
-🚇【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
@@ -5579,9 +5579,9 @@
       <c r="J77" s="3" t="inlineStr">
         <is>
           <t>★ 九龙土瓜湾核心大型重建标杆住区
-🚇【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈</t>
+【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
@@ -5645,9 +5645,9 @@
       <c r="J78" s="3" t="inlineStr">
         <is>
           <t>★ 九龙城联合道18号核心成熟板块
-🚇【轨交】步行约 7 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
+【轨交】步行约 7 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
+【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -5711,15 +5711,15 @@
       <c r="J79" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东核心北角英皇道绝佳占位
-🚇【轨交】步行约 3 分钟即达港铁炮台山站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
+【轨交】步行约 3 分钟即达港铁炮台山站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L79" s="3" t="inlineStr">
@@ -5777,15 +5777,15 @@
       <c r="J80" s="3" t="inlineStr">
         <is>
           <t>★ 港岛北角核心步行1-2分钟达北角站
-🚇【轨交】步行约 2 分钟即达港铁北角站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+【轨交】步行约 2 分钟即达港铁北角站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L80" s="3" t="inlineStr">
@@ -5843,9 +5843,9 @@
       <c r="J81" s="3" t="inlineStr">
         <is>
           <t>★ 港岛核心天后站步行约3分钟
-🚇【轨交】步行约 3 分钟即达港铁天后站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
+【轨交】步行约 3 分钟即达港铁天后站（轨交通勤从容便捷）
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -5910,14 +5910,14 @@
         <is>
           <t>★ 港岛东北角继园街大型旗舰园林私邸
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 8 分钟即达港铁北角站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+【轨交】步行约 8 分钟即达港铁北角站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L82" s="3" t="inlineStr">
@@ -5976,14 +5976,14 @@
         <is>
           <t>★ 港岛东一线临海绝版地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 5 分钟即达港铁北角站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+【轨交】步行约 5 分钟即达港铁北角站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L83" s="3" t="inlineStr">
@@ -6042,14 +6042,14 @@
         <is>
           <t>★ 港岛东一线临海绝版地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 4 分钟即达港铁北角站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+【轨交】步行约 4 分钟即达港铁北角站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L84" s="3" t="inlineStr">
@@ -6108,14 +6108,14 @@
         <is>
           <t>★ 港岛东一线临海绝版地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 3 分钟即达港铁北角站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+【轨交】步行约 3 分钟即达港铁北角站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L85" s="3" t="inlineStr">
@@ -6173,9 +6173,9 @@
       <c r="J86" s="3" t="inlineStr">
         <is>
           <t>★ 中环半山己连拿利3号核心绝版地段
-🚇【轨交】步行约 9 分钟即达港铁中環站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+【轨交】步行约 9 分钟即达港铁中環站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -6240,14 +6240,14 @@
         <is>
           <t>★ 东半山司徒拔道18号低密显赫豪宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L87" s="3" t="inlineStr">
@@ -6305,15 +6305,15 @@
       <c r="J88" s="3" t="inlineStr">
         <is>
           <t>★ 东半山司徒拔道18号低密显赫豪宅
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L88" s="3" t="inlineStr">
@@ -6372,14 +6372,14 @@
         <is>
           <t>★ 中半山波老道21号香港顶奢豪宅标杆
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L89" s="3" t="inlineStr">
@@ -6437,15 +6437,15 @@
       <c r="J90" s="3" t="inlineStr">
         <is>
           <t>★ 薄扶林道138号独立洋房顶奢地标
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L90" s="3" t="inlineStr">
@@ -6503,9 +6503,9 @@
       <c r="J91" s="3" t="inlineStr">
         <is>
           <t>★ 港岛中环核心半山坚道黄金地段
-🚇【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -6570,14 +6570,14 @@
         <is>
           <t>★ 港岛西半山旭龢道42号显赫巅峰地段
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L92" s="3" t="inlineStr">
@@ -6635,9 +6635,9 @@
       <c r="J93" s="3" t="inlineStr">
         <is>
           <t>★ 地段稀缺
-🚇【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -6701,9 +6701,9 @@
       <c r="J94" s="3" t="inlineStr">
         <is>
           <t>★ 地段稀缺
-🚇【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -6767,15 +6767,15 @@
       <c r="J95" s="3" t="inlineStr">
         <is>
           <t>★ 西半山宝珊道23号极低密16席传世大宅
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L95" s="3" t="inlineStr">
@@ -6833,15 +6833,15 @@
       <c r="J96" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西半山罗便臣道23号传统名门腹地
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L96" s="3" t="inlineStr">
@@ -6900,14 +6900,14 @@
         <is>
           <t>★ 中半山波老道21号传世顶奢大宅第2期
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L97" s="3" t="inlineStr">
@@ -6966,9 +6966,9 @@
         <is>
           <t>★ 港岛西半山罗便臣道80号经典名牌豪宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 8 分钟即达港铁西營盤站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+【轨交】步行约 8 分钟即达港铁西營盤站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -7032,9 +7032,9 @@
       <c r="J99" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西核心枢纽与极速通勤
-🚇【轨交】步行约 3 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+【轨交】步行约 3 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -7098,9 +7098,9 @@
       <c r="J100" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西黄金地段步达坚尼地城站约2分钟
-🚇【轨交】步行约 2 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+【轨交】步行约 2 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
@@ -7164,9 +7164,9 @@
       <c r="J101" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西坚尼地城临海一线视野
-🚇【轨交】步行约 5 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+【轨交】步行约 5 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -7236,9 +7236,9 @@
       <c r="K102" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L102" s="3" t="inlineStr">
@@ -7296,15 +7296,15 @@
       <c r="J103" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区传统顶级显赫富豪圈
-🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K103" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L103" s="3" t="inlineStr">
@@ -7368,9 +7368,9 @@
       <c r="K104" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L104" s="3" t="inlineStr">
@@ -7428,15 +7428,15 @@
       <c r="J105" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区寿臣山顶级独立洋房群
-🚇【轨交】步行约 12 分钟即达港铁海洋公園站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+【轨交】步行约 12 分钟即达港铁海洋公園站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K105" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L105" s="3" t="inlineStr">
@@ -7494,15 +7494,15 @@
       <c r="J106" s="3" t="inlineStr">
         <is>
           <t>★ 浅水湾道108号极度珍罕独立海景洋房
-🛍️【商业】邻近/周边1.5km聚合The Pulse等大型地标商圈
+️【商业】邻近/周边1.5km聚合The Pulse等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K106" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L106" s="3" t="inlineStr">
@@ -7566,9 +7566,9 @@
       </c>
       <c r="K107" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L107" s="3" t="inlineStr">
@@ -7626,15 +7626,15 @@
       <c r="J108" s="3" t="inlineStr">
         <is>
           <t>★ 香港山顶聂歌信山道亚洲顶奢楼王地标
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K108" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L108" s="3" t="inlineStr">
@@ -7693,14 +7693,14 @@
         <is>
           <t>★ 香港山顶聂歌信山道亚洲顶奢楼王地标
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K109" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L109" s="3" t="inlineStr">
@@ -7758,15 +7758,15 @@
       <c r="J110" s="3" t="inlineStr">
         <is>
           <t>★ 香港山顶加列山道12号巅峰独立洋房群
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K110" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L110" s="3" t="inlineStr">
@@ -7824,15 +7824,15 @@
       <c r="J111" s="3" t="inlineStr">
         <is>
           <t>★ 香港山顶宾吉道3号太古地产传世洋房
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K111" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L111" s="3" t="inlineStr">
@@ -7891,14 +7891,14 @@
         <is>
           <t>★ 太古地产港岛东柴湾罕见大型综合体
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
+【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K112" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L112" s="3" t="inlineStr">
@@ -7957,14 +7957,14 @@
         <is>
           <t>★ 渣甸山30年唯一罕见分层新盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合利园等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K113" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
+          <t>【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L113" s="3" t="inlineStr">
@@ -8022,9 +8022,9 @@
       <c r="J114" s="3" t="inlineStr">
         <is>
           <t>★ 港岛湾仔活道15号核心成熟地段
-🚇【轨交】步行约 9 分钟即达港铁灣仔站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合时代广场等大型地标商圈
+【轨交】步行约 9 分钟即达港铁灣仔站（轨交通勤从容便捷）
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合时代广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -8088,15 +8088,15 @@
       <c r="J115" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东核心西湾河站步行约4分钟
-🚇【轨交】步行约 4 分钟即达港铁西灣河站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
+【轨交】步行约 4 分钟即达港铁西灣河站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K115" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L115" s="3" t="inlineStr">
@@ -8154,15 +8154,15 @@
       <c r="J116" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东筲箕湾站步行约3分钟
-🚇【轨交】步行约 3 分钟即达港铁筲箕灣站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
+【轨交】步行约 3 分钟即达港铁筲箕灣站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K116" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L116" s="3" t="inlineStr">
@@ -8220,15 +8220,15 @@
       <c r="J117" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东核心筲箕湾东大街23号成熟商圈
-🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
+️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K117" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁筲箕灣站超12分钟，建议接驳小巴至地铁
-🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
+【交通】步行至最近港铁筲箕灣站超12分钟，建议接驳小巴至地铁
+【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L117" s="3" t="inlineStr">
@@ -8287,14 +8287,14 @@
         <is>
           <t>★ 薄扶林域多利道301号全海景现楼
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🛍️【商业】邻近/周边1.5km聚合数码港商场等大型地标商圈
+️【商业】邻近/周边1.5km聚合数码港商场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K118" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】步行至最近港铁堅尼地城站超12分钟，建议接驳小巴至地铁
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【交通】步行至最近港铁堅尼地城站超12分钟，建议接驳小巴至地铁
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L118" s="3" t="inlineStr">
@@ -8352,9 +8352,9 @@
       <c r="J119" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西营盘核心枢纽极速通达
-🚇【轨交】步行约 3 分钟即达港铁西營盤站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈</t>
+【轨交】步行约 3 分钟即达港铁西營盤站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈</t>
         </is>
       </c>
       <c r="K119" s="3" t="inlineStr">
@@ -8418,9 +8418,9 @@
       <c r="J120" s="3" t="inlineStr">
         <is>
           <t>★ 上环苏豪艺术区极低密顶奢私邸
-🚇【轨交】步行约 7 分钟即达港铁上環站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+【轨交】步行约 7 分钟即达港铁上環站（轨交通勤从容便捷）
+【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -8484,15 +8484,15 @@
       <c r="J121" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区赤柱村道纯正低密滨海豪宅
-🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K121" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L121" s="3" t="inlineStr">
@@ -8551,14 +8551,14 @@
         <is>
           <t>★ 港岛南区赤柱黄麻角道纯海景洋房及大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K122" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L122" s="3" t="inlineStr">
@@ -8616,15 +8616,15 @@
       <c r="J123" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区寿臣山道西稀缺纯独立洋房
-🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K123" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L123" s="3" t="inlineStr">
@@ -8682,15 +8682,15 @@
       <c r="J124" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区舂磡角海天径绝版5席独立大宅
-🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K124" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L124" s="3" t="inlineStr">
@@ -8748,15 +8748,15 @@
       <c r="J125" s="3" t="inlineStr">
         <is>
           <t>★ 赤柱半山环角道隐秘低密独栋纯墅区
-🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K125" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L125" s="3" t="inlineStr">
@@ -8815,14 +8815,14 @@
         <is>
           <t>★ 东半山大坑道339号传统显赫地段
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合利园等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K126" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L126" s="3" t="inlineStr">
@@ -8881,14 +8881,14 @@
         <is>
           <t>★ 港铁黄竹坑站上盖专属电梯直达
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K127" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L127" s="3" t="inlineStr">
@@ -8947,14 +8947,14 @@
         <is>
           <t>★ 港铁黄竹坑站上盖专属电梯直达
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K128" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L128" s="3" t="inlineStr">
@@ -9013,14 +9013,14 @@
         <is>
           <t>★ 港岛30年唯一新房地铁上盖
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K129" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L129" s="3" t="inlineStr">
@@ -9079,14 +9079,14 @@
         <is>
           <t>★ 港岛30年唯一新房地铁上盖
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K130" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L130" s="3" t="inlineStr">
@@ -9144,15 +9144,15 @@
       <c r="J131" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区鸭脷洲海旁水岸生活圈
-🚇【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K131" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L131" s="3" t="inlineStr">
@@ -9210,15 +9210,15 @@
       <c r="J132" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区鸭脷洲平澜街滨海水岸新盘
-🚇【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K132" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L132" s="3" t="inlineStr">
@@ -9277,14 +9277,14 @@
         <is>
           <t>★ 港铁黄竹坑站上盖港岛南岸第2期
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直连车站大堂）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直连车站大堂）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K133" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L133" s="3" t="inlineStr">
@@ -9343,14 +9343,14 @@
         <is>
           <t>★ 港铁黄竹坑站上盖港岛南岸首发旗舰项目
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座直连 THE SOUTHSIDE 商场与车站）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+【轨交】港铁黄竹坑站正上盖 / 直通（基座直连 THE SOUTHSIDE 商场与车站）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K134" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L134" s="3" t="inlineStr">
@@ -9409,14 +9409,14 @@
         <is>
           <t>★ 港铁黄竹坑站纯正铁路上盖
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K135" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L135" s="3" t="inlineStr">
@@ -9475,14 +9475,14 @@
         <is>
           <t>★ 港铁黄竹坑站纯正铁路上盖
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K136" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L136" s="3" t="inlineStr">
@@ -9540,14 +9540,14 @@
       <c r="J137" s="3" t="inlineStr">
         <is>
           <t>★ 港铁黄竹坑站上盖港岛南岸第5期
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
+【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
         </is>
       </c>
       <c r="K137" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -9606,15 +9606,15 @@
       <c r="J138" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区鸭脷洲海旁道一线游艇海景
-🚇【轨交】步行约 11 分钟即达港铁利東站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+【轨交】步行约 11 分钟即达港铁利東站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K138" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L138" s="3" t="inlineStr">
@@ -9672,15 +9672,15 @@
       <c r="J139" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区鸭脷洲大街步行约3分钟达利东站
-🚇【轨交】步行约 3 分钟即达港铁利東站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+【轨交】步行约 3 分钟即达港铁利東站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K139" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L139" s="3" t="inlineStr">
@@ -9738,15 +9738,15 @@
       <c r="J140" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东核心鲗鱼涌站步行约4分钟
-🚇【轨交】步行约 4 分钟即达港铁鰂魚涌站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
+【轨交】步行约 4 分钟即达港铁鰂魚涌站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K140" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L140" s="3" t="inlineStr">
@@ -9805,14 +9805,14 @@
         <is>
           <t>★ 港岛南区鸭脷洲一线临海现楼超级豪宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 7 分钟即达港铁海怡半島站（轨交通勤从容便捷）
+【轨交】步行约 7 分钟即达港铁海怡半島站（轨交通勤从容便捷）
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K141" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L141" s="3" t="inlineStr">
@@ -9870,15 +9870,15 @@
       <c r="J142" s="3" t="inlineStr">
         <is>
           <t>★ 跑马地桂芳街8号老牌名流核心区
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合利园等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K142" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L142" s="3" t="inlineStr">
@@ -9936,15 +9936,15 @@
       <c r="J143" s="3" t="inlineStr">
         <is>
           <t>★ 跑马地蓝塘道半山珍罕大型洋房群
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合利园等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K143" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
+【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L143" s="3" t="inlineStr">
@@ -10003,13 +10003,13 @@
         <is>
           <t>★ 港铁黄竹坑站上盖港岛南岸第5期
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
-🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
+【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
+️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
         </is>
       </c>
       <c r="K144" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10068,14 +10068,14 @@
       <c r="J145" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区承丰道16号海滨前排新地标
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
         </is>
       </c>
       <c r="K145" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10134,14 +10134,14 @@
       <c r="J146" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区承丰道16号海滨前排新地标
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
         </is>
       </c>
       <c r="K146" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10200,15 +10200,15 @@
       <c r="J147" s="3" t="inlineStr">
         <is>
           <t>★ 旺角核心洗衣街地段步入太子及旺角东双铁
-🚇【轨交】步行约 5 分钟即达港铁旺角東站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+【轨交】步行约 5 分钟即达港铁旺角東站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K147" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L147" s="3" t="inlineStr">
@@ -10267,14 +10267,14 @@
         <is>
           <t>★ 西南九龙绝版一线临海地王现楼
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
+️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K148" s="3" t="inlineStr">
         <is>
-          <t>🚇【交通】步行至最近港铁南昌站超12分钟，建议接驳小巴至地铁
-🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+          <t>【交通】步行至最近港铁南昌站超12分钟，建议接驳小巴至地铁
+【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L148" s="3" t="inlineStr">
@@ -10337,9 +10337,9 @@
       <c r="K149" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10403,9 +10403,9 @@
       <c r="K150" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10464,9 +10464,9 @@
       <c r="J151" s="3" t="inlineStr">
         <is>
           <t>★ 何文田自由道传统静谧高尚住宅地脉
-🚇【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
-🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈
+【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
+【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -10531,13 +10531,13 @@
         <is>
           <t>★ 太古地产港岛东柴湾罕见大型综合体
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈</t>
+【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈</t>
         </is>
       </c>
       <c r="K152" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）
+          <t>【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10597,13 +10597,13 @@
         <is>
           <t>★ 西南九龙绝版巨无霸大型发展区
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】步行约 10 分钟即达港铁長沙灣站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
+【轨交】步行约 10 分钟即达港铁長沙灣站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
         </is>
       </c>
       <c r="K153" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
+          <t>【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10662,14 +10662,14 @@
       <c r="J154" s="3" t="inlineStr">
         <is>
           <t>★ 九龙核心百万呎巨无霸都会重建
-🚇【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
+【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
         </is>
       </c>
       <c r="K154" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10728,15 +10728,15 @@
       <c r="J155" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东半山肇辉台6号极度低密传世私邸
-🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-🛍️【商业】邻近/周边1.5km聚合利东街等大型地标商圈
+【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+️【商业】邻近/周边1.5km聚合利东街等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K155" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L155" s="3" t="inlineStr">
@@ -10795,13 +10795,13 @@
         <is>
           <t>★ 港铁康城站临海前排一线开扬全海景
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
-🛍️【商业】连桥直达 The LOHAS 康城地标级商场</t>
+【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
+️【商业】连桥直达 The LOHAS 康城地标级商场</t>
         </is>
       </c>
       <c r="K156" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
+          <t>【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10861,13 +10861,13 @@
         <is>
           <t>★ 港铁康城站临海前排一线开扬全海景
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-🚇【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
-🛍️【商业】连桥直达 The LOHAS 康城地标级商场</t>
+【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
+️【商业】连桥直达 The LOHAS 康城地标级商场</t>
         </is>
       </c>
       <c r="K157" s="3" t="inlineStr">
         <is>
-          <t>🎓【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
+          <t>【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10926,14 +10926,14 @@
       <c r="J158" s="3" t="inlineStr">
         <is>
           <t>★ 北角核心繁华腹地与成熟商圈
-🚇【轨交】步行约 6 分钟即达港铁炮台山站（轨交通勤从容便捷）
-🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈</t>
+【轨交】步行约 6 分钟即达港铁炮台山站（轨交通勤从容便捷）
+️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈</t>
         </is>
       </c>
       <c r="K158" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）
+【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
@@ -10992,14 +10992,14 @@
       <c r="J159" s="3" t="inlineStr">
         <is>
           <t>★ 恒基西九龙市区更新全新力作
-🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈</t>
+️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈</t>
         </is>
       </c>
       <c r="K159" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-🚇【交通】步行至最近港铁太子站超12分钟，建议接驳小巴至地铁
-🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
+【交通】步行至最近港铁太子站超12分钟，建议接驳小巴至地铁
+【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>

</xml_diff>

<commit_message>
fix(map): resolve st. george's mansions single-quote escaping & calibrate Kai Tak runway transit to Kai Tak station
</commit_message>
<xml_diff>
--- a/导出方案项目描述库.xlsx
+++ b/导出方案项目描述库.xlsx
@@ -618,19 +618,21 @@
         <is>
           <t>★ 九龙塘龙庭里8号超级豪宅巅峰之作
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>步行约 1600米 (19分钟) 直达港铁九龍塘站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达九龍塘站
+港铁 3站达金钟 | 🚅 高铁 3站
+✈️ 机场约 26分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -683,20 +685,22 @@
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>★ 九龙塘龙庭里8号超级豪宅巅峰之作
-【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
+🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>步行约 1446米 (17分钟) 直达港铁九龍塘站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达九龍塘站
+港铁 3站达金钟 | 🚅 高铁 3站
+✈️ 机场约 26分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -749,20 +753,22 @@
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>★ 九龙塘龙庭里8号超级豪宅巅峰之作
-【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
+🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>步行约 1446米 (17分钟) 直达港铁九龍塘站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达九龍塘站
+港铁 3站达金钟 | 🚅 高铁 3站
+✈️ 机场约 26分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -815,20 +821,22 @@
       <c r="J5" s="3" t="inlineStr">
         <is>
           <t>★ 九龙塘广播道半山珍稀向南大宅
-🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🏡【社区】洋房与低密大宅复合庄园，享私家花园与低密专属会所
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>步行约 1403米 (16分钟) 直达港铁九龍塘站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达九龍塘站
+港铁 3站达金钟 | 🚅 高铁 3站
+✈️ 机场约 26分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -881,20 +889,22 @@
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>★ 九龙塘喇沙利道32-38号喇沙小学正对面
-【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>步行约 2297米 (27分钟) 直达港铁天后站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 3站达金钟 | 🚅 高铁 5站
+✈️ 机场约 26分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -947,20 +957,22 @@
       <c r="J7" s="3" t="inlineStr">
         <is>
           <t>★ 九龙笔架山半山龙驹道超级豪宅巅峰
-🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🏡【社区】洋房与低密大宅复合庄园，享私家花园与低密专属会所
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
-【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>步行约 2210米 (26分钟) 直达港铁長沙灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 7站达金钟 | 🚅 高铁 4站
+✈️ 机场约 25分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1014,19 +1026,21 @@
         <is>
           <t>★ 九龙站上盖香港地标级顶奢天际豪宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁九龙站正上盖 / 直通（直通圆方 ELEMENTS 与九龙站/柯士甸）
-️【商业】基座直通圆方 ELEMENTS 超大型购物中心
+🚇【轨交】港铁九龙站正上盖 / 直通（直通圆方 ELEMENTS 与九龙站/柯士甸）
+🛍️【商业】基座直通圆方 ELEMENTS 超大型购物中心
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>步行约 145米 (1分钟) 直达港铁九龍站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【九龍站正上盖 (圆方ELEMENTS直连)】
+港铁 1站达中环 | 🚅 高铁 直通
+✈️ 机场约 24分 | 🚘 深圳湾口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1079,20 +1093,22 @@
       <c r="J9" s="3" t="inlineStr">
         <is>
           <t>★ 何文田窝打老道黄金名校地段
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
+🚇【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>步行约 1070米 (12分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1145,9 +1161,9 @@
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>★ 太子道西核心地段新鸿基品质力作
-【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🚇【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1158,7 +1174,9 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>步行约 482米 (5分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 482米 (6分) 到旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1211,9 +1229,9 @@
       <c r="J11" s="3" t="inlineStr">
         <is>
           <t>★ 何文田自由道万科品质轻奢地标
-【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🚇【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1224,7 +1242,9 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>步行约 606米 (7分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 606米 (7分) 到旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1278,9 +1298,9 @@
         <is>
           <t>★ 何文田加多利山百年名门显赫地段
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🚇【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1291,7 +1311,9 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>步行约 724米 (8分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 724米 (9分) 到旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1345,19 +1367,21 @@
         <is>
           <t>★ 何文田核心传统豪宅区现楼大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>步行约 1165米 (14分钟) 直达港铁土瓜灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达土瓜灣站
+港铁 3站达金钟/中环 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1410,20 +1434,22 @@
       <c r="J14" s="3" t="inlineStr">
         <is>
           <t>★ 太子道西266号传统豪宅名门腹地
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
+🚇【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>步行约 1030米 (12分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1477,9 +1503,9 @@
         <is>
           <t>★ 何文田佛光街23号新鸿基巅峰豪宅标杆
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🚇【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1490,7 +1516,9 @@
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>步行约 459米 (5分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 459米 (6分) 到何文田站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1543,9 +1571,9 @@
       <c r="J16" s="3" t="inlineStr">
         <is>
           <t>★ 九龙顶尖34名校网黄金护城河
-【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🚇【轨交】步行约 9 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1556,7 +1584,9 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>步行约 740米 (8分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 740米 (9分) 到旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1609,20 +1639,22 @@
       <c r="J17" s="3" t="inlineStr">
         <is>
           <t>★ 太子道西279号极低密名门大宅
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
+🚇【交通】步行至最近港铁旺角東站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>步行约 1090米 (13分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1676,19 +1708,22 @@
         <is>
           <t>★ 港铁何文田站纯正铁路上盖绝版压轴大盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>步行约 386米 (4分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【何文田站正上盖 (专用电梯直达站厅)】
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1742,19 +1777,22 @@
         <is>
           <t>★ 港铁何文田站纯正铁路上盖绝版压轴大盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
+          <t>✨【五维全优】名校网 · 轨交直通 · 商业汇聚 · 大盘格局 · 即期交付，五维无显著量化短板</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>步行约 464米 (5分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【何文田站正上盖 (专用电梯直达站厅)】
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1808,9 +1846,9 @@
         <is>
           <t>★ 纯正铁路上盖双线枢纽极速通达
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
@@ -1821,7 +1859,9 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>步行约 368米 (4分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【何文田站正上盖 (专用电梯直达站厅)】
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1875,9 +1915,9 @@
         <is>
           <t>★ 纯正铁路上盖双线枢纽极速通达
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🚇【轨交】港铁何文田站正上盖 / 直通（专属高速客梯直通港铁站大堂）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -1888,7 +1928,9 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>步行约 292米 (3分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【何文田站正上盖 (专用电梯直达站厅)】
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -1941,20 +1983,22 @@
       <c r="J22" s="3" t="inlineStr">
         <is>
           <t>★ 何文田加多利山老牌名门贵胄地脉
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
+🚇【交通】步行至最近港铁土瓜灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>步行约 1115米 (13分钟) 直达港铁土瓜灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达土瓜灣站
+港铁 3站达金钟/中环 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -2007,9 +2051,9 @@
       <c r="J23" s="3" t="inlineStr">
         <is>
           <t>★ 何文田胜利道核心地段精品现楼
-【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🚇【轨交】步行约 7 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2020,7 +2064,9 @@
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>步行约 554米 (6分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 554米 (7分) 到旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -2073,9 +2119,9 @@
       <c r="J24" s="3" t="inlineStr">
         <is>
           <t>★ 窝打老道93号/太子道西交界传统豪宅核心
-【轨交】步行约 12 分钟即达港铁旺角東站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🚇【轨交】步行约 12 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2086,7 +2132,9 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>步行约 971米 (11分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 971米 (12分) 到旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -2139,20 +2187,22 @@
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>★ 加多利山与太子道西传统豪宅腹地
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁宋皇臺站超12分钟，建议接驳小巴至地铁</t>
+🚇【交通】步行至最近港铁宋皇臺站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>步行约 1045米 (12分钟) 直达港铁宋皇臺站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达宋皇臺站
+港铁 3站达金钟/中环 | 🚅 高铁 3站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -2206,19 +2256,21 @@
         <is>
           <t>★ 启德跑道区三面临海极佳水岸占位
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2272,19 +2324,21 @@
         <is>
           <t>★ 启德跑道区三面临海极佳水岸占位
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2338,9 +2392,9 @@
         <is>
           <t>★ 启德城中心现楼发售即买即住即收租
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 9 分钟即达港铁啟德站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈
+🚇【轨交】步行约 9 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2351,7 +2405,9 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>步行约 5-6 分钟直达港铁启德站（屯马线），两站即达钻石山/宋皇台，畅达全港</t>
+          <t>步行约 719米 (9分) 到啟德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2405,19 +2461,21 @@
         <is>
           <t>★ 启德跑道公园前排临海游艇景观
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2471,19 +2529,21 @@
         <is>
           <t>★ 启德跑道公园前排临海游艇景观
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2537,9 +2597,9 @@
         <is>
           <t>★ 启德城中心前排紧邻启德河与港铁站
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🚇【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2550,7 +2610,9 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>步行约 6-8 分钟直达港铁启德站（屯马线），立体路网贯穿港九</t>
+          <t>步行约 677米 (8分) 到啟德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2604,9 +2666,9 @@
         <is>
           <t>★ 启德城中心前排紧邻启德河与港铁站
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2617,7 +2679,9 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>步行约 6-8 分钟直达港铁启德站（屯马线），立体路网贯穿港九</t>
+          <t>步行约 607米 (7分) 到啟德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2671,9 +2735,9 @@
         <is>
           <t>★ 启德城中心前排紧邻启德河与港铁站
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🚇【轨交】步行约 8 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2684,7 +2748,9 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>步行约 6-8 分钟直达港铁启德站（屯马线），立体路网贯穿港九</t>
+          <t>步行约 643米 (8分) 到啟德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2738,9 +2804,9 @@
         <is>
           <t>★ 启德城中心前排与双重视觉地标
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2751,7 +2817,9 @@
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>步行约 5-7 分钟直达港铁启德站（屯马线），快速连通中环金钟及九龙东双CBD核心</t>
+          <t>步行约 557米 (7分) 到啟德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2804,9 +2872,9 @@
       <c r="J35" s="3" t="inlineStr">
         <is>
           <t>★ 启德城中心前排与双重视觉地标
-【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2817,7 +2885,9 @@
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>步行约 5-7 分钟直达港铁启德站（屯马线），快速连通中环金钟及九龙东双CBD核心</t>
+          <t>步行约 557米 (7分) 到啟德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2871,9 +2941,9 @@
         <is>
           <t>★ 启德城中心前排与双重视觉地标
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
+🚇【轨交】步行约 7 分钟即达港铁啟德站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合双子汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -2884,7 +2954,9 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>步行约 5-7 分钟直达港铁启德站（屯马线），快速连通中环金钟及九龙东双CBD核心</t>
+          <t>步行约 566米 (7分) 到啟德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -2938,19 +3010,21 @@
         <is>
           <t>★ 启德跑道区核心海滨大型旗舰热销盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3004,19 +3078,21 @@
         <is>
           <t>★ 启德跑道区核心海滨大型旗舰热销盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L38" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3070,19 +3146,21 @@
         <is>
           <t>★ 启德跑道区龙头前排绝对一线临海地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3136,9 +3214,9 @@
         <is>
           <t>★ 启德唯一全天候无缝直达地铁新盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
+🚇【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -3149,7 +3227,9 @@
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>港铁启德站无缝上盖核心枢纽，地下街直通车站及超甲级商厦AIRSIDE/双子汇；自驾经中九龙干线极速通达全港</t>
+          <t>港铁【啟德站正上盖 (地下街直通车站)】
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3203,9 +3283,9 @@
         <is>
           <t>★ 启德唯一全天候无缝直达地铁新盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
+🚇【轨交】港铁启德站正上盖 / 直通（全天候地下街直通启德站与AIRSIDE）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】下楼直达 AIRSIDE 与双子汇地标级商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -3216,7 +3296,9 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>港铁启德站无缝上盖核心枢纽，地下街直通车站及超甲级商厦AIRSIDE/双子汇；自驾经中九龙干线极速通达全港</t>
+          <t>港铁【啟德站正上盖 (地下街直通车站)】
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3270,19 +3352,21 @@
         <is>
           <t>★ 启德跑道区最前排半岛位龙头地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议接驳穿梭巴士至港铁啟德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>港铁【九龍站正上盖 (圆方ELEMENTS直连)】
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3335,20 +3419,22 @@
       <c r="J43" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区最前排半岛位龙头地王
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+🚇【交通】建议接驳穿梭巴士至港铁啟德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>港铁【九龍站正上盖 (圆方ELEMENTS直连)】
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3402,19 +3488,21 @@
         <is>
           <t>★ 启德跑道区最前排半岛位龙头地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议接驳穿梭巴士至港铁啟德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>港铁【九龍站正上盖 (圆方ELEMENTS直连)】
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3468,19 +3556,21 @@
         <is>
           <t>★ 启德跑道区三面环海绝佳占位
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3534,19 +3624,21 @@
         <is>
           <t>★ 启德跑道区三面环海绝佳占位
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3599,20 +3691,22 @@
       <c r="J47" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区三面环海绝佳占位
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3665,20 +3759,22 @@
       <c r="J48" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区一线临海龙头
-🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🏡【社区】洋房与低密大宅复合庄园，享私家花园与低密专属会所
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3731,20 +3827,22 @@
       <c r="J49" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区首发大型地标住宅承丰道21号
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3798,19 +3896,21 @@
         <is>
           <t>★ 启德跑道区核心承丰里2号双子地标
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L50" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3864,19 +3964,21 @@
         <is>
           <t>★ 启德跑道区前排龙头一线临海大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L51" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3930,19 +4032,21 @@
         <is>
           <t>★ 启德跑道区前排龙头一线临海大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L52" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -3996,19 +4100,21 @@
         <is>
           <t>★ 启德跑道区前排龙头一线临海大宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -4061,20 +4167,22 @@
       <c r="J54" s="3" t="inlineStr">
         <is>
           <t>★ 九龙佐敦德成街2号闹中取静绝佳地段
-【轨交】步行约 2 分钟即达港铁佐敦站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合美丽华广场等大型地标商圈
+🚇【轨交】步行约 2 分钟即达港铁佐敦站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合美丽华广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L54" s="3" t="inlineStr">
         <is>
-          <t>步行约 163米 (2分钟) 直达港铁佐敦站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 163米 (2分) 到佐敦站
+港铁 2站达金钟 | 🚅 高铁 1站
+✈️ 机场约 28分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -4127,20 +4235,22 @@
       <c r="J55" s="3" t="inlineStr">
         <is>
           <t>★ 九龙繁华腹地界限街交通枢纽
-【轨交】步行约 10 分钟即达港铁深水埗站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合西九龙中心等大型地标商圈
+🚇【轨交】步行约 10 分钟即达港铁深水埗站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合西九龙中心等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>步行约 836米 (10分钟) 直达港铁深水埗站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 836米 (10分) 到深水埗站
+港铁 6站达金钟 | 🚅 高铁 3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -4193,20 +4303,22 @@
       <c r="J56" s="3" t="inlineStr">
         <is>
           <t>★ 太子道西核心地脉步入双铁立体枢纽
-【轨交】步行约 4 分钟即达港铁太子站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈</t>
+🚇【轨交】步行约 4 分钟即达港铁太子站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈</t>
         </is>
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L56" s="3" t="inlineStr">
         <is>
-          <t>步行约 345米 (4分钟) 直达港铁太子站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 345米 (4分) 到太子站
+港铁 5站达金钟 | 🚅 高铁 3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -4260,19 +4372,21 @@
         <is>
           <t>★ 西九龙核心大角咀大型艺文商业街区
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
+🚇【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L57" s="3" t="inlineStr">
         <is>
-          <t>步行约 909米 (10分钟) 直达港铁奧運站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 909米 (11分) 到奧運站
+港铁 2-4站达核心 | 🚅 高铁 2-3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -4326,19 +4440,21 @@
         <is>
           <t>★ 西九龙核心大角咀大型艺文商业街区
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
+🚇【轨交】步行约 11 分钟即达港铁奧運站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L58" s="3" t="inlineStr">
         <is>
-          <t>步行约 909米 (10分钟) 直达港铁奧運站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 909米 (11分) 到奧運站
+港铁 2-4站达核心 | 🚅 高铁 2-3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -4391,20 +4507,22 @@
       <c r="J59" s="3" t="inlineStr">
         <is>
           <t>★ 西九龙大角咀核心生活圈交通极速通达
-【轨交】步行约 10 分钟即达港铁旺角站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
+🚇【轨交】步行约 10 分钟即达港铁旺角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
         <is>
-          <t>步行约 819米 (9分钟) 直达港铁旺角站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 819米 (10分) 到旺角站
+港铁 4站达金钟 | 🚅 高铁 2站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -4457,20 +4575,22 @@
       <c r="J60" s="3" t="inlineStr">
         <is>
           <t>★ 九龙油麻地核心商圈全新精品住宅
-【轨交】步行约 6 分钟即达港铁油麻地站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合朗豪坊等大型地标商圈</t>
+🚇【轨交】步行约 6 分钟即达港铁油麻地站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合朗豪坊等大型地标商圈</t>
         </is>
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属31校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L60" s="3" t="inlineStr">
         <is>
-          <t>步行约 509米 (6分钟) 直达港铁油麻地站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 509米 (6分) 到油麻地站
+港铁 3站达金钟 | 🚅 高铁 1站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -4529,14 +4649,16 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
-【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】步行至最近港铁長沙灣站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr">
         <is>
-          <t>步行约 2071米 (24分钟) 直达港铁長沙灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 7站达金钟 | 🚅 高铁 4站
+✈️ 机场约 25分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -4589,20 +4711,22 @@
       <c r="J62" s="3" t="inlineStr">
         <is>
           <t>★ 九龙塘又一村低密传世尊贵名邸
-️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
+🛍️【商业】邻近/周边1.5km聚合又一城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁
-【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+🚇【交通】步行至最近港铁九龍塘站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L62" s="3" t="inlineStr">
         <is>
-          <t>步行约 1019米 (12分钟) 直达港铁九龍塘站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达九龍塘站
+港铁 3站达金钟 | 🚅 高铁 3站
+✈️ 机场约 25分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -4655,20 +4779,22 @@
       <c r="J63" s="3" t="inlineStr">
         <is>
           <t>★ 红磡核心三轨枢纽立体交通网络
-【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
+🚇【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L63" s="3" t="inlineStr">
         <is>
-          <t>步行约 550米 (6分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 550米 (7分) 到何文田站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -4721,20 +4847,22 @@
       <c r="J64" s="3" t="inlineStr">
         <is>
           <t>★ 九龙核心百万呎巨无霸都会重建
-【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
+🚇【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L64" s="3" t="inlineStr">
         <is>
-          <t>步行约 414米 (5分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 414米 (5分) 到何文田站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -4787,20 +4915,22 @@
       <c r="J65" s="3" t="inlineStr">
         <is>
           <t>★ 九龙核心百万呎巨无霸都会重建
-【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
+🚇【轨交】步行约 6 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L65" s="3" t="inlineStr">
         <is>
-          <t>步行约 471米 (5分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 471米 (6分) 到何文田站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -4853,20 +4983,22 @@
       <c r="J66" s="3" t="inlineStr">
         <is>
           <t>★ 九龙土瓜湾高山道公园旁清幽地段
-【轨交】步行约 6 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
+🚇【轨交】步行约 6 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L66" s="3" t="inlineStr">
         <is>
-          <t>步行约 536米 (6分钟) 直达港铁土瓜灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 536米 (6分) 到土瓜灣站
+港铁 3站达金钟/中环 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -4919,20 +5051,22 @@
       <c r="J67" s="3" t="inlineStr">
         <is>
           <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
-【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+🚇【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L67" s="3" t="inlineStr">
         <is>
-          <t>步行约 724米 (8分钟) 直达港铁土瓜灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 724米 (9分) 到土瓜灣站
+港铁 3站达金钟/中环 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -4985,20 +5119,22 @@
       <c r="J68" s="3" t="inlineStr">
         <is>
           <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
-【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
+🚇【轨交】步行约 9 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
         </is>
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L68" s="3" t="inlineStr">
         <is>
-          <t>步行约 724米 (8分钟) 直达港铁土瓜灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 724米 (9分) 到土瓜灣站
+港铁 3站达金钟/中环 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -5051,20 +5187,22 @@
       <c r="J69" s="3" t="inlineStr">
         <is>
           <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
-【轨交】步行约 8 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+🚇【轨交】步行约 8 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L69" s="3" t="inlineStr">
         <is>
-          <t>步行约 648米 (7分钟) 直达港铁土瓜灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 648米 (8分) 到土瓜灣站
+港铁 3站达金钟/中环 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -5117,20 +5255,22 @@
       <c r="J70" s="3" t="inlineStr">
         <is>
           <t>★ 九龙红磡/土瓜湾大型千伙综合体地标
-【轨交】步行约 7 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+🚇【轨交】步行约 7 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L70" s="3" t="inlineStr">
         <is>
-          <t>步行约 598米 (7分钟) 直达港铁土瓜灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 598米 (7分) 到土瓜灣站
+港铁 3站达金钟/中环 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -5183,20 +5323,22 @@
       <c r="J71" s="3" t="inlineStr">
         <is>
           <t>★ 红磡核心枢纽珍罕999年期地契
-【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
+🚇【轨交】步行约 7 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
         </is>
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L71" s="3" t="inlineStr">
         <is>
-          <t>步行约 599米 (7分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 599米 (7分) 到何文田站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -5250,19 +5392,21 @@
         <is>
           <t>★ 西南九龙绝版巨无霸大型发展区
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 10 分钟即达港铁荔枝角站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
+🚇【轨交】步行约 10 分钟即达港铁荔枝角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
         </is>
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
+          <t>🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L72" s="3" t="inlineStr">
         <is>
-          <t>步行约 874米 (10分钟) 直达港铁荔枝角站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 874米 (10分) 到荔枝角站
+港铁 8站达金钟 | 🚅 高铁 4站
+✈️ 机场约 22分 | 🚘 深圳湾口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -5316,19 +5460,21 @@
         <is>
           <t>★ 港铁南昌站纯正铁路上盖双线枢纽
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁南昌站正上盖 / 直通（基座 V Walk 直通南昌站双铁枢纽）
-️【商业】基座直连近 30 万呎 V Walk 大型综合商场
+🚇【轨交】港铁南昌站正上盖 / 直通（基座 V Walk 直通南昌站双铁枢纽）
+🛍️【商业】基座直连近 30 万呎 V Walk 大型综合商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L73" s="3" t="inlineStr">
         <is>
-          <t>港铁南昌站正上盖物业（东涌线与屯马线双线交汇），一站直达西九龙高铁站及香港站（中环），极速贯通全港核心</t>
+          <t>港铁【南昌站正上盖 (V Walk商场直通)】
+港铁 2站达中环 | 🚅 高铁 1站
+✈️ 机场约 22分 | 🚘 深圳湾口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -5382,19 +5528,21 @@
         <is>
           <t>★ 西南九龙绝版一线临海地王现楼
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
+🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁南昌站超12分钟，建议接驳小巴至地铁
-【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L74" s="3" t="inlineStr">
         <is>
-          <t>步行约 1374米 (16分钟) 直达港铁南昌站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 22分 | 🚘 深圳湾口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -5447,9 +5595,9 @@
       <c r="J75" s="3" t="inlineStr">
         <is>
           <t>★ 九龙城宋皇台站步行约4-5分钟
-【轨交】步行约 5 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
-【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
+🚇【轨交】步行约 5 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
@@ -5460,7 +5608,9 @@
       </c>
       <c r="L75" s="3" t="inlineStr">
         <is>
-          <t>步行约 406米 (4分钟) 直达港铁宋皇臺站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 406米 (5分) 到宋皇臺站
+港铁 3站达金钟/中环 | 🚅 高铁 3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -5513,9 +5663,9 @@
       <c r="J76" s="3" t="inlineStr">
         <is>
           <t>★ 九龙土瓜湾核心大型重建标杆住区
-【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
+🚇【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合爱民广场等大型地标商圈</t>
         </is>
       </c>
       <c r="K76" s="3" t="inlineStr">
@@ -5526,7 +5676,9 @@
       </c>
       <c r="L76" s="3" t="inlineStr">
         <is>
-          <t>步行约 418米 (5分钟) 直达港铁土瓜灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 418米 (5分) 到土瓜灣站
+港铁 3站达金钟/中环 | 🚅 高铁 2站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -5579,9 +5731,9 @@
       <c r="J77" s="3" t="inlineStr">
         <is>
           <t>★ 九龙土瓜湾核心大型重建标杆住区
-【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈</t>
+🚇【轨交】步行约 5 分钟即达港铁土瓜灣站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合启德体育园零售馆等大型地标商圈</t>
         </is>
       </c>
       <c r="K77" s="3" t="inlineStr">
@@ -5592,7 +5744,9 @@
       </c>
       <c r="L77" s="3" t="inlineStr">
         <is>
-          <t>步行约 421米 (5分钟) 直达港铁土瓜灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 421米 (5分) 到土瓜灣站
+港铁 3站达金钟/中环 | 🚅 高铁 2站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -5645,9 +5799,9 @@
       <c r="J78" s="3" t="inlineStr">
         <is>
           <t>★ 九龙城联合道18号核心成熟板块
-【轨交】步行约 7 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
-【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
+🚇【轨交】步行约 7 分钟即达港铁宋皇臺站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 41 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合Mikiki等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -5658,7 +5812,9 @@
       </c>
       <c r="L78" s="3" t="inlineStr">
         <is>
-          <t>步行约 559米 (6分钟) 直达港铁宋皇臺站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 559米 (7分) 到宋皇臺站
+港铁 3站达金钟/中环 | 🚅 高铁 3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -5711,20 +5867,22 @@
       <c r="J79" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东核心北角英皇道绝佳占位
-【轨交】步行约 3 分钟即达港铁炮台山站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
+🚇【轨交】步行约 3 分钟即达港铁炮台山站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L79" s="3" t="inlineStr">
         <is>
-          <t>步行约 280米 (3分钟) 直达港铁炮台山站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 280米 (3分) 到炮台山站
+港铁 4站达金钟 | 🚅 高铁 5站
+✈️ 机场约 36分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -5777,20 +5935,22 @@
       <c r="J80" s="3" t="inlineStr">
         <is>
           <t>★ 港岛北角核心步行1-2分钟达北角站
-【轨交】步行约 2 分钟即达港铁北角站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🚇【轨交】步行约 2 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L80" s="3" t="inlineStr">
         <is>
-          <t>步行约 140米 (1分钟) 直达港铁北角站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 140米 (2分) 到北角站
+港铁 5站达金钟 | 🚅 高铁 6站
+✈️ 机场约 36分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -5843,9 +6003,9 @@
       <c r="J81" s="3" t="inlineStr">
         <is>
           <t>★ 港岛核心天后站步行约3分钟
-【轨交】步行约 3 分钟即达港铁天后站（轨交通勤从容便捷）
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
+🚇【轨交】步行约 3 分钟即达港铁天后站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合皇室堡等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -5856,7 +6016,9 @@
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t>步行约 282米 (3分钟) 直达港铁天后站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 282米 (3分) 到天后站
+港铁 3站达金钟 | 🚅 高铁 5站
+✈️ 机场约 36分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -5910,19 +6072,21 @@
         <is>
           <t>★ 港岛东北角继园街大型旗舰园林私邸
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 8 分钟即达港铁北角站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🚇【轨交】步行约 8 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>步行约 661米 (7分钟) 直达港铁北角站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 661米 (8分) 到北角站
+港铁 5站达金钟 | 🚅 高铁 6站
+✈️ 机场约 36分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -5976,19 +6140,21 @@
         <is>
           <t>★ 港岛东一线临海绝版地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 5 分钟即达港铁北角站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🚇【轨交】步行约 5 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L83" s="3" t="inlineStr">
         <is>
-          <t>步行约 407米 (4分钟) 直达港铁北角站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 407米 (5分) 到北角站
+港铁 5站达金钟 | 🚅 高铁 6站
+✈️ 机场约 36分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6042,19 +6208,21 @@
         <is>
           <t>★ 港岛东一线临海绝版地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 4 分钟即达港铁北角站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🚇【轨交】步行约 4 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L84" s="3" t="inlineStr">
         <is>
-          <t>步行约 306米 (3分钟) 直达港铁北角站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 306米 (4分) 到北角站
+港铁 5站达金钟 | 🚅 高铁 6站
+✈️ 机场约 36分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6108,19 +6276,21 @@
         <is>
           <t>★ 港岛东一线临海绝版地王
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 3 分钟即达港铁北角站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
+🚇【轨交】步行约 3 分钟即达港铁北角站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L85" s="3" t="inlineStr">
         <is>
-          <t>步行约 274米 (3分钟) 直达港铁北角站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 274米 (3分) 到北角站
+港铁 5站达金钟 | 🚅 高铁 6站
+✈️ 机场约 36分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6173,9 +6343,9 @@
       <c r="J86" s="3" t="inlineStr">
         <is>
           <t>★ 中环半山己连拿利3号核心绝版地段
-【轨交】步行约 9 分钟即达港铁中環站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🚇【轨交】步行约 9 分钟即达港铁中環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -6186,7 +6356,9 @@
       </c>
       <c r="L86" s="3" t="inlineStr">
         <is>
-          <t>步行约 734米 (8分钟) 直达港铁中環站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 734米 (9分) 到中環站
+港铁 中环直达 | 🚅 高铁 1站
+✈️ 机场约 32分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6239,20 +6411,22 @@
       <c r="J87" s="3" t="inlineStr">
         <is>
           <t>★ 东半山司徒拔道18号低密显赫豪宅
-🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
+🏡【社区】洋房与低密大宅复合庄园，享私家花园与低密专属会所
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L87" s="3" t="inlineStr">
         <is>
-          <t>步行约 1708米 (20分钟) 直达港铁灣仔站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6305,20 +6479,22 @@
       <c r="J88" s="3" t="inlineStr">
         <is>
           <t>★ 东半山司徒拔道18号低密显赫豪宅
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
-          <t>步行约 1708米 (20分钟) 直达港铁灣仔站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6372,19 +6548,21 @@
         <is>
           <t>★ 中半山波老道21号香港顶奢豪宅标杆
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L89" s="3" t="inlineStr">
         <is>
-          <t>步行约 1709米 (20分钟) 直达港铁金鐘站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 金钟直达 | 🚅 高铁 2站
+✈️ 机场约 32分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6437,20 +6615,22 @@
       <c r="J90" s="3" t="inlineStr">
         <is>
           <t>★ 薄扶林道138号独立洋房顶奢地标
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K90" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L90" s="3" t="inlineStr">
         <is>
-          <t>步行约 1152米 (13分钟) 直达港铁香港大學站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达香港大學站
+港铁 3站达中环 | 🚅 高铁 4站
+✈️ 机场约 32分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6503,9 +6683,9 @@
       <c r="J91" s="3" t="inlineStr">
         <is>
           <t>★ 港岛中环核心半山坚道黄金地段
-【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🚇【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -6516,7 +6696,9 @@
       </c>
       <c r="L91" s="3" t="inlineStr">
         <is>
-          <t>步行约 891米 (10分钟) 直达港铁上環站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 891米 (11分) 到上環站
+港铁 1站达中环 | 🚅 高铁 2站
+✈️ 机场约 32分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6570,19 +6752,21 @@
         <is>
           <t>★ 港岛西半山旭龢道42号显赫巅峰地段
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L92" s="3" t="inlineStr">
         <is>
-          <t>步行约 1021米 (12分钟) 直达港铁香港大學站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达香港大學站
+港铁 3站达中环 | 🚅 高铁 4站
+✈️ 机场约 32分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6635,9 +6819,9 @@
       <c r="J93" s="3" t="inlineStr">
         <is>
           <t>★ 地段稀缺
-【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🚇【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -6648,7 +6832,9 @@
       </c>
       <c r="L93" s="3" t="inlineStr">
         <is>
-          <t>步行约 947米 (11分钟) 直达港铁上環站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 947米 (11分) 到上環站
+港铁 1站达中环 | 🚅 高铁 2站
+✈️ 机场约 32分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6701,9 +6887,9 @@
       <c r="J94" s="3" t="inlineStr">
         <is>
           <t>★ 地段稀缺
-【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🚇【轨交】步行约 11 分钟即达港铁上環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -6714,7 +6900,9 @@
       </c>
       <c r="L94" s="3" t="inlineStr">
         <is>
-          <t>步行约 947米 (11分钟) 直达港铁上環站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 947米 (11分) 到上環站
+港铁 1站达中环 | 🚅 高铁 2站
+✈️ 机场约 32分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6767,20 +6955,22 @@
       <c r="J95" s="3" t="inlineStr">
         <is>
           <t>★ 西半山宝珊道23号极低密16席传世大宅
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L95" s="3" t="inlineStr">
         <is>
-          <t>步行约 1241米 (14分钟) 直达港铁香港大學站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达香港大學站
+港铁 3站达中环 | 🚅 高铁 4站
+✈️ 机场约 32分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6833,20 +7023,22 @@
       <c r="J96" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西半山罗便臣道23号传统名门腹地
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L96" s="3" t="inlineStr">
         <is>
-          <t>步行约 1146米 (13分钟) 直达港铁上環站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达上環站
+港铁 1站达中环 | 🚅 高铁 2站
+✈️ 机场约 32分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6900,19 +7092,21 @@
         <is>
           <t>★ 中半山波老道21号传世顶奢大宅第2期
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合太古广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L97" s="3" t="inlineStr">
         <is>
-          <t>步行约 1764米 (21分钟) 直达港铁金鐘站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 金钟直达 | 🚅 高铁 2站
+✈️ 机场约 32分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -6966,9 +7160,9 @@
         <is>
           <t>★ 港岛西半山罗便臣道80号经典名牌豪宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 8 分钟即达港铁西營盤站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🚇【轨交】步行约 8 分钟即达港铁西營盤站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -6979,7 +7173,9 @@
       </c>
       <c r="L98" s="3" t="inlineStr">
         <is>
-          <t>步行约 650米 (7分钟) 直达港铁西營盤站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 650米 (8分) 到西營盤站
+港铁 2站达中环 | 🚅 高铁 3站
+✈️ 机场约 32分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7032,9 +7228,9 @@
       <c r="J99" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西核心枢纽与极速通勤
-【轨交】步行约 3 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🚇【轨交】步行约 3 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -7045,7 +7241,9 @@
       </c>
       <c r="L99" s="3" t="inlineStr">
         <is>
-          <t>步行约 281米 (3分钟) 直达港铁堅尼地城站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 281米 (3分) 到堅尼地城站
+港铁 4站达中环 | 🚅 高铁 5站
+✈️ 机场约 30分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7098,9 +7296,9 @@
       <c r="J100" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西黄金地段步达坚尼地城站约2分钟
-【轨交】步行约 2 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🚇【轨交】步行约 2 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
@@ -7111,7 +7309,9 @@
       </c>
       <c r="L100" s="3" t="inlineStr">
         <is>
-          <t>步行约 151米 (1分钟) 直达港铁堅尼地城站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 151米 (2分) 到堅尼地城站
+港铁 4站达中环 | 🚅 高铁 5站
+✈️ 机场约 30分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7164,9 +7364,9 @@
       <c r="J101" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西坚尼地城临海一线视野
-【轨交】步行约 5 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🚇【轨交】步行约 5 分钟即达港铁堅尼地城站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -7177,7 +7377,9 @@
       </c>
       <c r="L101" s="3" t="inlineStr">
         <is>
-          <t>步行约 410米 (4分钟) 直达港铁堅尼地城站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 410米 (5分) 到堅尼地城站
+港铁 4站达中环 | 🚅 高铁 5站
+✈️ 机场约 30分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7230,20 +7432,22 @@
       <c r="J102" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区大潭白笔山道一线纯独立海景洋房
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K102" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L102" s="3" t="inlineStr">
         <is>
-          <t>步行约 5466米 (65分钟) 直达港铁柴灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 12站达中环 | 🚅 高铁 13站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7296,20 +7500,22 @@
       <c r="J103" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区传统顶级显赫富豪圈
-️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K103" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L103" s="3" t="inlineStr">
         <is>
-          <t>步行约 1110米 (13分钟) 直达港铁海洋公園站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达海洋公園站
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 40分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -7368,14 +7574,16 @@
       <c r="K104" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L104" s="3" t="inlineStr">
         <is>
-          <t>步行约 3164米 (38分钟) 直达港铁海洋公園站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 40分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -7428,20 +7636,22 @@
       <c r="J105" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区寿臣山顶级独立洋房群
-【轨交】步行约 12 分钟即达港铁海洋公園站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🚇【轨交】步行约 12 分钟即达港铁海洋公園站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K105" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L105" s="3" t="inlineStr">
         <is>
-          <t>步行约 996米 (12分钟) 直达港铁海洋公園站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 996米 (12分) 到海洋公園站
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 40分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -7494,20 +7704,22 @@
       <c r="J106" s="3" t="inlineStr">
         <is>
           <t>★ 浅水湾道108号极度珍罕独立海景洋房
-️【商业】邻近/周边1.5km聚合The Pulse等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🛍️【商业】邻近/周边1.5km聚合The Pulse等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K106" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L106" s="3" t="inlineStr">
         <is>
-          <t>步行约 3408米 (40分钟) 直达港铁海洋公園站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 40分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -7560,20 +7772,22 @@
       <c r="J107" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区深水湾径超级隐秘纯豪宅
-🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
+🏡【社区】洋房与低密大宅复合庄园，享私家花园与低密专属会所
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K107" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L107" s="3" t="inlineStr">
         <is>
-          <t>步行约 1685米 (20分钟) 直达港铁海洋公園站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 30分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -7626,20 +7840,22 @@
       <c r="J108" s="3" t="inlineStr">
         <is>
           <t>★ 香港山顶聂歌信山道亚洲顶奢楼王地标
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合合和商场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K108" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L108" s="3" t="inlineStr">
         <is>
-          <t>步行约 3647米 (43分钟) 直达港铁灣仔站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 40分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7692,20 +7908,22 @@
       <c r="J109" s="3" t="inlineStr">
         <is>
           <t>★ 香港山顶聂歌信山道亚洲顶奢楼王地标
-🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🏡【社区】洋房与低密大宅复合庄园，享私家花园与低密专属会所
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K109" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L109" s="3" t="inlineStr">
         <is>
-          <t>步行约 3696米 (44分钟) 直达港铁灣仔站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 40分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7758,20 +7976,22 @@
       <c r="J110" s="3" t="inlineStr">
         <is>
           <t>★ 香港山顶加列山道12号巅峰独立洋房群
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K110" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L110" s="3" t="inlineStr">
         <is>
-          <t>步行约 3334米 (40分钟) 直达港铁中環站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 中环直达 | 🚅 高铁 1站
+✈️ 机场约 40分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7824,20 +8044,22 @@
       <c r="J111" s="3" t="inlineStr">
         <is>
           <t>★ 香港山顶宾吉道3号太古地产传世洋房
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合山顶广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K111" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L111" s="3" t="inlineStr">
         <is>
-          <t>步行约 4143米 (49分钟) 直达港铁金鐘站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 金钟直达 | 🚅 高铁 2站
+✈️ 机场约 40分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7891,19 +8113,21 @@
         <is>
           <t>★ 太古地产港岛东柴湾罕见大型综合体
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
+🚇【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K112" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L112" s="3" t="inlineStr">
         <is>
-          <t>步行约 945米 (11分钟) 直达港铁柴灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 945米 (12分) 到柴灣站
+港铁 12站达中环 | 🚅 高铁 13站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -7957,19 +8181,21 @@
         <is>
           <t>★ 渣甸山30年唯一罕见分层新盘
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K113" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁天后站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L113" s="3" t="inlineStr">
         <is>
-          <t>步行约 1809米 (21分钟) 直达港铁天后站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 3站达金钟 | 🚅 高铁 5站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -8022,9 +8248,9 @@
       <c r="J114" s="3" t="inlineStr">
         <is>
           <t>★ 港岛湾仔活道15号核心成熟地段
-【轨交】步行约 9 分钟即达港铁灣仔站（轨交通勤从容便捷）
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合时代广场等大型地标商圈
+🚇【轨交】步行约 9 分钟即达港铁灣仔站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合时代广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -8035,7 +8261,9 @@
       </c>
       <c r="L114" s="3" t="inlineStr">
         <is>
-          <t>步行约 715米 (8分钟) 直达港铁灣仔站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 715米 (9分) 到灣仔站
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 32分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -8088,20 +8316,22 @@
       <c r="J115" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东核心西湾河站步行约4分钟
-【轨交】步行约 4 分钟即达港铁西灣河站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
+🚇【轨交】步行约 4 分钟即达港铁西灣河站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K115" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L115" s="3" t="inlineStr">
         <is>
-          <t>步行约 339米 (4分钟) 直达港铁西灣河站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 339米 (4分) 到西灣河站
+港铁 8站达中环 | 🚅 高铁 9站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -8154,20 +8384,22 @@
       <c r="J116" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东筲箕湾站步行约3分钟
-【轨交】步行约 3 分钟即达港铁筲箕灣站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
+🚇【轨交】步行约 3 分钟即达港铁筲箕灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K116" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L116" s="3" t="inlineStr">
         <is>
-          <t>步行约 262米 (3分钟) 直达港铁筲箕灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 262米 (3分) 到筲箕灣站
+港铁 9站达中环 | 🚅 高铁 10站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -8220,20 +8452,22 @@
       <c r="J117" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东核心筲箕湾东大街23号成熟商圈
-️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
+🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K117" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁筲箕灣站超12分钟，建议接驳小巴至地铁
-【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
+🚇【交通】步行至最近港铁筲箕灣站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L117" s="3" t="inlineStr">
         <is>
-          <t>步行约 1073米 (12分钟) 直达港铁筲箕灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达筲箕灣站
+港铁 9站达中环 | 🚅 高铁 10站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -8287,19 +8521,21 @@
         <is>
           <t>★ 薄扶林域多利道301号全海景现楼
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-️【商业】邻近/周边1.5km聚合数码港商场等大型地标商圈
+🛍️【商业】邻近/周边1.5km聚合数码港商场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K118" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁堅尼地城站超12分钟，建议接驳小巴至地铁
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L118" s="3" t="inlineStr">
         <is>
-          <t>步行约 1541米 (18分钟) 直达港铁堅尼地城站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -8352,20 +8588,22 @@
       <c r="J119" s="3" t="inlineStr">
         <is>
           <t>★ 港岛西营盘核心枢纽极速通达
-【轨交】步行约 3 分钟即达港铁西營盤站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈</t>
+🚇【轨交】步行约 3 分钟即达港铁西營盤站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合西宝城等大型地标商圈
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K119" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧</t>
         </is>
       </c>
       <c r="L119" s="3" t="inlineStr">
         <is>
-          <t>步行约 234米 (2分钟) 直达港铁西營盤站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 234米 (3分) 到西營盤站
+港铁 2站达中环 | 🚅 高铁 3站
+✈️ 机场约 28分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -8418,9 +8656,9 @@
       <c r="J120" s="3" t="inlineStr">
         <is>
           <t>★ 上环苏豪艺术区极低密顶奢私邸
-【轨交】步行约 7 分钟即达港铁上環站（轨交通勤从容便捷）
-【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
+🚇【轨交】步行约 7 分钟即达港铁上環站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 11 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合置地广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -8431,7 +8669,9 @@
       </c>
       <c r="L120" s="3" t="inlineStr">
         <is>
-          <t>步行约 555米 (6分钟) 直达港铁上環站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 555米 (7分) 到上環站
+港铁 1站达中环 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 深圳湾口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -8484,20 +8724,22 @@
       <c r="J121" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区赤柱村道纯正低密滨海豪宅
-️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K121" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L121" s="3" t="inlineStr">
         <is>
-          <t>步行约 7824米 (93分钟) 直达港铁柴灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 12站达中环 | 🚅 高铁 13站
+✈️ 机场约 40分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -8550,20 +8792,22 @@
       <c r="J122" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区赤柱黄麻角道纯海景洋房及大宅
-🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🏡【社区】洋房与低密大宅复合庄园，享私家花园与低密专属会所
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K122" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L122" s="3" t="inlineStr">
         <is>
-          <t>步行约 10184米 (122分钟) 直达港铁柴灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 12站达中环 | 🚅 高铁 13站
+✈️ 机场约 40分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -8616,20 +8860,22 @@
       <c r="J123" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区寿臣山道西稀缺纯独立洋房
-️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K123" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L123" s="3" t="inlineStr">
         <is>
-          <t>步行约 6946米 (83分钟) 直达港铁海洋公園站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 40分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -8682,20 +8928,22 @@
       <c r="J124" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区舂磡角海天径绝版5席独立大宅
-️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K124" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L124" s="3" t="inlineStr">
         <is>
-          <t>步行约 6345米 (76分钟) 直达港铁海洋公園站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 40分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -8748,20 +8996,22 @@
       <c r="J125" s="3" t="inlineStr">
         <is>
           <t>★ 赤柱半山环角道隐秘低密独栋纯墅区
-️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🛍️【商业】邻近/周边1.5km聚合赤柱广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K125" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L125" s="3" t="inlineStr">
         <is>
-          <t>步行约 6842米 (82分钟) 直达港铁海洋公園站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 40分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -8815,19 +9065,21 @@
         <is>
           <t>★ 东半山大坑道339号传统显赫地段
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K126" s="3" t="inlineStr">
         <is>
-          <t>【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L126" s="3" t="inlineStr">
         <is>
-          <t>步行约 2992米 (35分钟) 直达港铁銅鑼灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 40分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -8881,19 +9133,21 @@
         <is>
           <t>★ 港铁黄竹坑站上盖专属电梯直达
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K127" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L127" s="3" t="inlineStr">
         <is>
-          <t>步行约 183米 (2分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -8947,19 +9201,21 @@
         <is>
           <t>★ 港铁黄竹坑站上盖专属电梯直达
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（专属电梯直达港铁黄竹坑站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】准现楼阶段（短期即将收楼入伙，确定性高）</t>
         </is>
       </c>
       <c r="K128" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L128" s="3" t="inlineStr">
         <is>
-          <t>步行约 98米 (1分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9013,19 +9269,21 @@
         <is>
           <t>★ 港岛30年唯一新房地铁上盖
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K129" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L129" s="3" t="inlineStr">
         <is>
-          <t>步行约 33米 (0分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9079,19 +9337,21 @@
         <is>
           <t>★ 港岛30年唯一新房地铁上盖
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座直连港铁黄竹坑站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K130" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L130" s="3" t="inlineStr">
         <is>
-          <t>步行约 81米 (1分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9144,20 +9404,22 @@
       <c r="J131" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区鸭脷洲海旁水岸生活圈
-【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🚇【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K131" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L131" s="3" t="inlineStr">
         <is>
-          <t>步行约 473米 (5分钟) 直达港铁利東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 473米 (6分) 到利東站
+港铁 3站达金钟 | 🚅 高铁 5站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9210,20 +9472,22 @@
       <c r="J132" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区鸭脷洲平澜街滨海水岸新盘
-【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🚇【轨交】步行约 6 分钟即达港铁利東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K132" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L132" s="3" t="inlineStr">
         <is>
-          <t>步行约 533米 (6分钟) 直达港铁利東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 533米 (6分) 到利東站
+港铁 3站达金钟 | 🚅 高铁 5站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9277,19 +9541,21 @@
         <is>
           <t>★ 港铁黄竹坑站上盖港岛南岸第2期
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直连车站大堂）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直连车站大堂）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K133" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L133" s="3" t="inlineStr">
         <is>
-          <t>港铁黄竹坑站正上盖港岛南岸（南港岛线），两站直达金钟核心枢纽，商场THE SOUTHSIDE无缝直连</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9343,19 +9609,21 @@
         <is>
           <t>★ 港铁黄竹坑站上盖港岛南岸首发旗舰项目
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁黄竹坑站正上盖 / 直通（基座直连 THE SOUTHSIDE 商场与车站）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座直连 THE SOUTHSIDE 商场与车站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K134" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L134" s="3" t="inlineStr">
         <is>
-          <t>步行约 501米 (6分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9409,19 +9677,21 @@
         <is>
           <t>★ 港铁黄竹坑站纯正铁路上盖
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K135" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L135" s="3" t="inlineStr">
         <is>
-          <t>步行约 414米 (5分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9475,19 +9745,21 @@
         <is>
           <t>★ 港铁黄竹坑站纯正铁路上盖
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座专属电梯直通港铁站）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K136" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L136" s="3" t="inlineStr">
         <is>
-          <t>步行约 381米 (4分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9540,20 +9812,22 @@
       <c r="J137" s="3" t="inlineStr">
         <is>
           <t>★ 港铁黄竹坑站上盖港岛南岸第5期
-【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
         </is>
       </c>
       <c r="K137" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L137" s="3" t="inlineStr">
         <is>
-          <t>步行约 366米 (4分钟) 直达港铁黃竹坑站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9606,20 +9880,22 @@
       <c r="J138" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区鸭脷洲海旁道一线游艇海景
-【轨交】步行约 11 分钟即达港铁利東站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🚇【轨交】步行约 11 分钟即达港铁利東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K138" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L138" s="3" t="inlineStr">
         <is>
-          <t>步行约 892米 (10分钟) 直达港铁利東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 892米 (11分) 到利東站
+港铁 3站达金钟 | 🚅 高铁 5站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9672,20 +9948,22 @@
       <c r="J139" s="3" t="inlineStr">
         <is>
           <t>★ 港岛南区鸭脷洲大街步行约3分钟达利东站
-【轨交】步行约 3 分钟即达港铁利東站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
+🚇【轨交】步行约 3 分钟即达港铁利東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合The Southside等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K139" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L139" s="3" t="inlineStr">
         <is>
-          <t>步行约 282米 (3分钟) 直达港铁利東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 282米 (3分) 到利東站
+港铁 3站达金钟 | 🚅 高铁 5站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9738,20 +10016,22 @@
       <c r="J140" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东核心鲗鱼涌站步行约4分钟
-【轨交】步行约 4 分钟即达港铁鰂魚涌站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
+🚇【轨交】步行约 4 分钟即达港铁鰂魚涌站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合太古城中心等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K140" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L140" s="3" t="inlineStr">
         <is>
-          <t>步行约 362米 (4分钟) 直达港铁鰂魚涌站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 362米 (4分) 到鰂魚涌站
+港铁 6站达金钟 | 🚅 高铁 7站
+✈️ 机场约 36分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -9805,19 +10085,21 @@
         <is>
           <t>★ 港岛南区鸭脷洲一线临海现楼超级豪宅
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 7 分钟即达港铁海怡半島站（轨交通勤从容便捷）
+🚇【轨交】步行约 7 分钟即达港铁海怡半島站（轨交通勤从容便捷）
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K141" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L141" s="3" t="inlineStr">
         <is>
-          <t>步行约 594米 (7分钟) 直达港铁海怡半島站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 594米 (7分) 到海怡半島站
+港铁 4站达金钟 | 🚅 高铁 6站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -9870,20 +10152,22 @@
       <c r="J142" s="3" t="inlineStr">
         <is>
           <t>★ 跑马地桂芳街8号老牌名流核心区
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K142" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
+🚇【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L142" s="3" t="inlineStr">
         <is>
-          <t>步行约 1891米 (22分钟) 直达港铁銅鑼灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -9936,20 +10220,22 @@
       <c r="J143" s="3" t="inlineStr">
         <is>
           <t>★ 跑马地蓝塘道半山珍罕大型洋房群
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合利园等大型地标商圈
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利园等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K143" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
+          <t>🚇【交通】步行至最近港铁銅鑼灣站超12分钟，建议接驳小巴至地铁</t>
         </is>
       </c>
       <c r="L143" s="3" t="inlineStr">
         <is>
-          <t>步行约 1824米 (21分钟) 直达港铁銅鑼灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -10003,19 +10289,21 @@
         <is>
           <t>★ 港铁黄竹坑站上盖港岛南岸第5期
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
-️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
+🚇【轨交】港铁黄竹坑站正上盖 / 直通（基座无缝直通黄竹坑站大堂）
+🛍️【商业】基座直达 51 万呎 THE SOUTHSIDE 地标级商场</t>
         </is>
       </c>
       <c r="K144" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+          <t>🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L144" s="3" t="inlineStr">
         <is>
-          <t>港铁黄竹坑站正上盖港岛南岸（南港岛线），两站直达金钟核心枢纽，商场THE SOUTHSIDE无缝直连</t>
+          <t>港铁【黃竹坑站正上盖 (商场THE SOUTHSIDE直连)】
+港铁 2站达金钟 | 🚅 高铁 4站
+✈️ 机场约 34分 | 🚘 深圳湾口岸 38分*</t>
         </is>
       </c>
     </row>
@@ -10068,20 +10356,22 @@
       <c r="J145" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区承丰道16号海滨前排新地标
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
         </is>
       </c>
       <c r="K145" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】建议接驳小巴至港铁啟德站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L145" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -10134,20 +10424,22 @@
       <c r="J146" s="3" t="inlineStr">
         <is>
           <t>★ 启德跑道区承丰道16号海滨前排新地标
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队</t>
         </is>
       </c>
       <c r="K146" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】建议接驳小巴至港铁牛頭角站（日常出行依赖专线接驳）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
+🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L146" s="3" t="inlineStr">
         <is>
-          <t>专线巴士约 5-8 分钟直达港铁启德站/宋皇台站；自驾经中九龙干线极速贯通全港</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 30分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -10200,20 +10492,22 @@
       <c r="J147" s="3" t="inlineStr">
         <is>
           <t>★ 旺角核心洗衣街地段步入太子及旺角东双铁
-【轨交】步行约 5 分钟即达港铁旺角東站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
+🚇【轨交】步行约 5 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合MOKO 新世纪广场等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K147" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L147" s="3" t="inlineStr">
         <is>
-          <t>步行约 407米 (4分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 407米 (5分) 到旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -10266,20 +10560,22 @@
       <c r="J148" s="3" t="inlineStr">
         <is>
           <t>★ 西南九龙绝版一线临海地王现楼
-🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
+🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K148" s="3" t="inlineStr">
         <is>
-          <t>【交通】步行至最近港铁南昌站超12分钟，建议接驳小巴至地铁
-【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
+          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
+🚇【交通】建议搭乘承丰道专线小巴约5-8分钟接驳至港铁启德站（日常出行依赖专线接驳）
+🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）</t>
         </is>
       </c>
       <c r="L148" s="3" t="inlineStr">
         <is>
-          <t>步行约 1247米 (15分钟) 直达港铁南昌站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 跑道穿梭巴士约 5-8分 直达启德站
+港铁 4站达金钟/中环 | 🚅 高铁 4站
+✈️ 机场约 22分 | 🚘 深圳湾口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -10331,21 +10627,23 @@
       </c>
       <c r="J149" s="3" t="inlineStr">
         <is>
-          <t>★ 港岛大潭白笔山道18号经典滨海独立洋房</t>
+          <t>★ 港岛大潭白笔山道18号经典滨海独立洋房
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K149" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
-⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L149" s="3" t="inlineStr">
         <is>
-          <t>步行约 6034米 (72分钟) 直达港铁柴灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 12站达中环 | 🚅 高铁 13站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -10397,21 +10695,23 @@
       </c>
       <c r="J150" s="3" t="inlineStr">
         <is>
-          <t>★ 港岛大潭白笔山道18号经典滨海独立洋房</t>
+          <t>★ 港岛大潭白笔山道18号经典滨海独立洋房
+🏡【社区】顶级纯独立洋房聚落，享私家花园泳池与至高隐逸私密
+🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K150" s="3" t="inlineStr">
         <is>
-          <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
-【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
-️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈
-⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
+          <t>🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾
+🎓【校网】非传统四大名校网（所属18校网，升学建议搭配优质私立或国际学校）
+🛍️【商业】周边1.5km暂无大型商业综合体，日常集中消费依赖外溢商圈</t>
         </is>
       </c>
       <c r="L150" s="3" t="inlineStr">
         <is>
-          <t>步行约 5395米 (64分钟) 直达港铁柴灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚘 专属车队约 6-8分 接驳核心港铁
+港铁 12站达中环 | 🚅 高铁 13站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -10464,9 +10764,9 @@
       <c r="J151" s="3" t="inlineStr">
         <is>
           <t>★ 何文田自由道传统静谧高尚住宅地脉
-【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
-【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈
+🚇【轨交】步行约 6 分钟即达港铁旺角東站（轨交通勤从容便捷）
+🎓【名校】全港顶尖 34 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合T.O.P等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
@@ -10477,7 +10777,9 @@
       </c>
       <c r="L151" s="3" t="inlineStr">
         <is>
-          <t>步行约 499米 (6分钟) 直达港铁旺角東站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 499米 (6分) 到旺角東站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -10531,19 +10833,21 @@
         <is>
           <t>★ 太古地产港岛东柴湾罕见大型综合体
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈</t>
+🚇【轨交】步行约 12 分钟即达港铁柴灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合杏花新城等大型地标商圈</t>
         </is>
       </c>
       <c r="K152" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）
+          <t>🎓【校网】非传统四大名校网（所属16校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L152" s="3" t="inlineStr">
         <is>
-          <t>步行约 945米 (11分钟) 直达港铁柴灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 945米 (12分) 到柴灣站
+港铁 12站达中环 | 🚅 高铁 13站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -10597,19 +10901,21 @@
         <is>
           <t>★ 西南九龙绝版巨无霸大型发展区
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】步行约 10 分钟即达港铁長沙灣站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
+🚇【轨交】步行约 10 分钟即达港铁長沙灣站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合V Walk等大型地标商圈</t>
         </is>
       </c>
       <c r="K153" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
+          <t>🎓【校网】非传统四大名校网（所属40校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L153" s="3" t="inlineStr">
         <is>
-          <t>步行约 817米 (10分钟) 直达港铁長沙灣站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 817米 (10分) 到長沙灣站
+港铁 7站达金钟 | 🚅 高铁 4站
+✈️ 机场约 22分 | 🚘 深圳湾口岸 28分*</t>
         </is>
       </c>
     </row>
@@ -10662,20 +10968,22 @@
       <c r="J154" s="3" t="inlineStr">
         <is>
           <t>★ 九龙核心百万呎巨无霸都会重建
-【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
+🚇【轨交】步行约 5 分钟即达港铁何文田站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合黄埔天地等大型地标商圈</t>
         </is>
       </c>
       <c r="K154" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属35校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L154" s="3" t="inlineStr">
         <is>
-          <t>步行约 424米 (5分钟) 直达港铁何文田站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 424米 (5分) 到何文田站
+港铁 2站达金钟 | 🚅 高铁 2站
+✈️ 机场约 28分 | 🚘 皇岗口岸 32分*</t>
         </is>
       </c>
     </row>
@@ -10728,20 +11036,22 @@
       <c r="J155" s="3" t="inlineStr">
         <is>
           <t>★ 港岛东半山肇辉台6号极度低密传世私邸
-【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
-️【商业】邻近/周边1.5km聚合利东街等大型地标商圈
+🎓【名校】全港顶尖 12 名校网，享传统公立名校优质升学梯队
+🛍️【商业】邻近/周边1.5km聚合利东街等大型地标商圈
 🔑【交付】现楼发售（即买即住 / 即时收租，实景所见即所得）</t>
         </is>
       </c>
       <c r="K155" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
+🚇【交通】地处低密私密地脉无就近步行地铁站，依赖接驳小巴或自驾</t>
         </is>
       </c>
       <c r="L155" s="3" t="inlineStr">
         <is>
-          <t>步行约 1065米 (13分钟) 直达港铁灣仔站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达灣仔站
+港铁 1站达金钟 | 🚅 高铁 3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -10795,19 +11105,21 @@
         <is>
           <t>★ 港铁康城站临海前排一线开扬全海景
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
-️【商业】连桥直达 The LOHAS 康城地标级商场</t>
+🚇【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
+🛍️【商业】连桥直达 The LOHAS 康城地标级商场</t>
         </is>
       </c>
       <c r="K156" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
+          <t>🎓【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L156" s="3" t="inlineStr">
         <is>
-          <t>步行约 305米 (3分钟) 直达港铁康城站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【康城站正上盖 (商场The LOHAS直通)】
+港铁 7站达中环 | 🚅 高铁 8站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -10861,19 +11173,21 @@
         <is>
           <t>★ 港铁康城站临海前排一线开扬全海景
 🏡【社区】多座组团地标大盘，配备大型度假式综合会所与园林
-【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
-️【商业】连桥直达 The LOHAS 康城地标级商场</t>
+🚇【轨交】港铁康城站正上盖 / 直通（室内全天候天桥直通 The LOHAS 与康城站）
+🛍️【商业】连桥直达 The LOHAS 康城地标级商场</t>
         </is>
       </c>
       <c r="K157" s="3" t="inlineStr">
         <is>
-          <t>【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
+          <t>🎓【校网】非传统四大名校网（所属95校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L157" s="3" t="inlineStr">
         <is>
-          <t>步行约 277米 (3分钟) 直达港铁康城站，轨交干线高效直通中环/九龙核心</t>
+          <t>港铁【康城站正上盖 (商场The LOHAS直通)】
+港铁 7站达中环 | 🚅 高铁 8站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -10926,20 +11240,22 @@
       <c r="J158" s="3" t="inlineStr">
         <is>
           <t>★ 北角核心繁华腹地与成熟商圈
-【轨交】步行约 6 分钟即达港铁炮台山站（轨交通勤从容便捷）
-️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈</t>
+🚇【轨交】步行约 6 分钟即达港铁炮台山站（轨交通勤从容便捷）
+🛍️【商业】邻近/周边1.5km聚合北角汇等大型地标商圈</t>
         </is>
       </c>
       <c r="K158" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）
+🎓【校网】非传统四大名校网（所属14校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L158" s="3" t="inlineStr">
         <is>
-          <t>步行约 496米 (6分钟) 直达港铁炮台山站，轨交干线高效直通中环/九龙核心</t>
+          <t>步行约 496米 (6分) 到炮台山站
+港铁 4站达金钟 | 🚅 高铁 5站
+✈️ 机场约 36分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>
@@ -10992,20 +11308,22 @@
       <c r="J159" s="3" t="inlineStr">
         <is>
           <t>★ 恒基西九龙市区更新全新力作
-️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈</t>
+🛍️【商业】邻近/周边1.5km聚合奥海城等大型地标商圈</t>
         </is>
       </c>
       <c r="K159" s="3" t="inlineStr">
         <is>
           <t>🏢【社区】属单幢精致物业，公用绿化及大型会所相对小巧
-【交通】步行至最近港铁太子站超12分钟，建议接驳小巴至地铁
-【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
+🚇【交通】步行至最近港铁太子站超12分钟，建议接驳小巴至地铁
+🎓【校网】非传统四大名校网（所属32校网，升学建议搭配优质私立或国际学校）
 ⏳【交付】属预售楼花阶段（预计交付周期超1年，需等待工程竣工）</t>
         </is>
       </c>
       <c r="L159" s="3" t="inlineStr">
         <is>
-          <t>步行约 1028米 (12分钟) 直达港铁太子站，轨交干线高效直通中环/九龙核心</t>
+          <t>🚌 专线小巴约 3-5分 直达太子站
+港铁 5站达金钟 | 🚅 高铁 3站
+✈️ 机场约 30分 | 🚘 皇岗口岸 35分*</t>
         </is>
       </c>
     </row>

</xml_diff>